<commit_message>
Use PDF allocation ratios and fix overseas manager section
</commit_message>
<xml_diff>
--- a/outputs/blf-monthly-disclosure/勞工退休基金月度揭露_可持續更新.xlsx
+++ b/outputs/blf-monthly-disclosure/勞工退休基金月度揭露_可持續更新.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板" sheetId="1" r:id="Rd9d690488bf34826"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板(美元)" sheetId="2" r:id="R712cff793c084fe7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度資產配置" sheetId="3" r:id="Rfdf1439ccf4d4651"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國內委外明細" sheetId="4" r:id="R28e19e45e77a40cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國外委外明細" sheetId="5" r:id="Rab2d8c31d9c643a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次彙總" sheetId="6" r:id="Rc4cb1f0ab88d473b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業者彙總" sheetId="7" r:id="R9698cc44cd9941e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新說明" sheetId="8" r:id="R500c691197ed41d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料品質檢核" sheetId="9" r:id="Reccff047312b4c61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板" sheetId="1" r:id="R669daac13ad74f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板(美元)" sheetId="2" r:id="R33a107dc429342d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度資產配置" sheetId="3" r:id="R038d41fa085c48ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國內委外明細" sheetId="4" r:id="R90f8d2ff99c0436a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國外委外明細" sheetId="5" r:id="R98c7add857854f5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次彙總" sheetId="6" r:id="R95dcd709b20e4a79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業者彙總" sheetId="7" r:id="R655147c3abff4a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新說明" sheetId="8" r:id="Rd797195441a049c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料品質檢核" sheetId="9" r:id="R00327db2d15443fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3375,7 +3375,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R905a40ff0de945f2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8bcbffc68bdd42c7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3405,7 +3405,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re8e84e7c91bb4e87"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re347ddf758a443cf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3435,7 +3435,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raff075e4e6a94ebf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8327dbd615e5436d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3465,7 +3465,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5651826484714962"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc802eff804884510"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3495,7 +3495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4e97b0b8b3bf4f98"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra942c1960ef0439b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3530,7 +3530,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R966977981ce74a40"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ref3eb68545f84288"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3560,7 +3560,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R045feacbf19c4d28"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R06365c72ff574aa6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3590,7 +3590,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9adaabd040074666"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8fabfa9601cf43b8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3620,7 +3620,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf00fa6fc94bc4cd1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3b8271fb31fc4e07"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3650,7 +3650,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf92c1442f732439f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9e842dc2cb7e4bfb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3685,7 +3685,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R583f8382e45e4b4c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc1c31b906090403b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3715,7 +3715,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re0d1abcd5d5e44a7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R73cbe4e5c09a4c57"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3745,7 +3745,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra9089d7219a54419"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Reda42996294f4f1d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3775,7 +3775,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd6c668e20cfd4394"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3ca6cd30a901413c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4374,36 +4374,36 @@
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="W12" s="50" t="n">
-        <x:f>IFERROR(B19/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.08009049818080267</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.08010000000000002</x:v>
       </x:c>
       <x:c r="X12" t="str">
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="Y12" s="50" t="n">
-        <x:f>IFERROR(C19/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.20294689334834715</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.2029</x:v>
       </x:c>
       <x:c r="Z12" t="str">
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="AA12" s="50" t="n">
-        <x:f>IFERROR(D19/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.09830773672574242</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0983</x:v>
       </x:c>
       <x:c r="AB12" t="str">
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="AC12" s="50" t="n">
-        <x:f>IFERROR(E19/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.04795105887019382</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.048</x:v>
       </x:c>
       <x:c r="AD12" t="str">
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="AE12" s="50" t="n">
-        <x:f>IFERROR(F19/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.09545607450479587</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.107325</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4434,35 +4434,35 @@
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="W13" s="50" t="n">
-        <x:f>IFERROR(B20/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X13" t="str">
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="Y13" s="50" t="n">
-        <x:f>IFERROR(C20/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z13" t="str">
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="AA13" s="50" t="n">
-        <x:f>IFERROR(D20/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB13" t="str">
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="AC13" s="50" t="n">
-        <x:f>IFERROR(E20/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD13" t="str">
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="AE13" s="50" t="n">
-        <x:f>IFERROR(F20/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4494,36 +4494,36 @@
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="W14" s="50" t="n">
-        <x:f>IFERROR(B21/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.025587121477121857</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.025600000000000005</x:v>
       </x:c>
       <x:c r="X14" t="str">
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="Y14" s="50" t="n">
-        <x:f>IFERROR(C21/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.06119948492201287</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.061200000000000004</x:v>
       </x:c>
       <x:c r="Z14" t="str">
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="AA14" s="50" t="n">
-        <x:f>IFERROR(D21/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.026053089900866026</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.026099999999999998</x:v>
       </x:c>
       <x:c r="AB14" t="str">
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="AC14" s="50" t="n">
-        <x:f>IFERROR(E21/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.0174561842083449</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0174</x:v>
       </x:c>
       <x:c r="AD14" t="str">
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="AE14" s="50" t="n">
-        <x:f>IFERROR(F21/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.029328348097442464</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.032575</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -4554,36 +4554,36 @@
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="W15" s="50" t="n">
-        <x:f>IFERROR(B22/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.04215323484379305</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.042100000000000005</x:v>
       </x:c>
       <x:c r="X15" t="str">
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="Y15" s="50" t="n">
-        <x:f>IFERROR(C22/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z15" t="str">
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="AA15" s="50" t="n">
-        <x:f>IFERROR(D22/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.04390044141522057</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.043899999999999995</x:v>
       </x:c>
       <x:c r="AB15" t="str">
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="AC15" s="50" t="n">
-        <x:f>IFERROR(E22/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.06906982845758472</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0691</x:v>
       </x:c>
       <x:c r="AD15" t="str">
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="AE15" s="50" t="n">
-        <x:f>IFERROR(F22/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.03969409795326574</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.038775</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -4614,36 +4614,36 @@
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="W16" s="50" t="n">
-        <x:f>IFERROR(B23/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X16" t="str">
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="Y16" s="50" t="n">
-        <x:f>IFERROR(C23/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.07236318107912533</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0724</x:v>
       </x:c>
       <x:c r="Z16" t="str">
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="AA16" s="50" t="n">
-        <x:f>IFERROR(D23/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB16" t="str">
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="AC16" s="50" t="n">
-        <x:f>IFERROR(E23/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD16" t="str">
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="AE16" s="50" t="n">
-        <x:f>IFERROR(F23/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.00894763287013099</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0181</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -4674,36 +4674,36 @@
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="W17" s="50" t="n">
-        <x:f>IFERROR(B24/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X17" t="str">
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="Y17" s="50" t="n">
-        <x:f>IFERROR(C24/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z17" t="str">
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="AA17" s="50" t="n">
-        <x:f>IFERROR(D24/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.0009475554586620803</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0009</x:v>
       </x:c>
       <x:c r="AB17" t="str">
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="AC17" s="50" t="n">
-        <x:f>IFERROR(E24/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD17" t="str">
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="AE17" s="50" t="n">
-        <x:f>IFERROR(F24/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.0001615598458113894</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.000225</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -4734,36 +4734,36 @@
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="W18" s="50" t="n">
-        <x:f>IFERROR(B25/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X18" t="str">
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="Y18" s="50" t="n">
-        <x:f>IFERROR(C25/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z18" t="str">
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="AA18" s="50" t="n">
-        <x:f>IFERROR(D25/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.0004527288739017158</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0005</x:v>
       </x:c>
       <x:c r="AB18" t="str">
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="AC18" s="50" t="n">
-        <x:f>IFERROR(E25/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD18" t="str">
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="AE18" s="50" t="n">
-        <x:f>IFERROR(F25/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.00007719105662184733</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.000125</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -4794,36 +4794,36 @@
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="W19" s="50" t="n">
-        <x:f>IFERROR(B26/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X19" t="str">
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="Y19" s="50" t="n">
-        <x:f>IFERROR(C26/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z19" t="str">
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="AA19" s="50" t="n">
-        <x:f>IFERROR(D26/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.02049930093134865</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.020499999999999997</x:v>
       </x:c>
       <x:c r="AB19" t="str">
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="AC19" s="50" t="n">
-        <x:f>IFERROR(E26/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD19" t="str">
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="AE19" s="50" t="n">
-        <x:f>IFERROR(F26/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.0034951662907268884</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.005124999999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -4854,36 +4854,36 @@
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="W20" s="50" t="n">
-        <x:f>IFERROR(B27/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.052170363275692376</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0522</x:v>
       </x:c>
       <x:c r="X20" t="str">
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="Y20" s="50" t="n">
-        <x:f>IFERROR(C27/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.07214944417511744</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0721</x:v>
       </x:c>
       <x:c r="Z20" t="str">
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="AA20" s="50" t="n">
-        <x:f>IFERROR(D27/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.3098279686321394</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.3098</x:v>
       </x:c>
       <x:c r="AB20" t="str">
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="AC20" s="50" t="n">
-        <x:f>IFERROR(E27/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.26199942183961406</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.262</x:v>
       </x:c>
       <x:c r="AD20" t="str">
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="AE20" s="50" t="n">
-        <x:f>IFERROR(F27/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.11771113488688957</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.174025</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -4914,36 +4914,36 @@
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="W21" s="50" t="n">
-        <x:f>IFERROR(B12/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.12075808373788141</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.12080000000000002</x:v>
       </x:c>
       <x:c r="X21" t="str">
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="Y21" s="50" t="n">
-        <x:f>IFERROR(C12/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.02481659353415637</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0248</x:v>
       </x:c>
       <x:c r="Z21" t="str">
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="AA21" s="50" t="n">
-        <x:f>IFERROR(D12/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.11512469419841453</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1151</x:v>
       </x:c>
       <x:c r="AB21" t="str">
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="AC21" s="50" t="n">
-        <x:f>IFERROR(E12/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.1224335921276509</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.12240000000000001</x:v>
       </x:c>
       <x:c r="AD21" t="str">
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="AE21" s="50" t="n">
-        <x:f>IFERROR(F12/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.10808734407200997</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.095775</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -4974,36 +4974,36 @@
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="W22" s="50" t="n">
-        <x:f>IFERROR(B13/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.01407056112684972</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.014100000000000001</x:v>
       </x:c>
       <x:c r="X22" t="str">
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="Y22" s="50" t="n">
-        <x:f>IFERROR(C13/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.018345364867298538</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0184</x:v>
       </x:c>
       <x:c r="Z22" t="str">
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="AA22" s="50" t="n">
-        <x:f>IFERROR(D13/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.06043946381637647</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0604</x:v>
       </x:c>
       <x:c r="AB22" t="str">
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="AC22" s="50" t="n">
-        <x:f>IFERROR(E13/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.06682090781757392</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0668</x:v>
       </x:c>
       <x:c r="AD22" t="str">
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="AE22" s="50" t="n">
-        <x:f>IFERROR(F13/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.027316675295284924</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.039925</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -5034,36 +5034,36 @@
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="W23" s="50" t="n">
-        <x:f>IFERROR(B14/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.007729314146437791</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.007700000000000001</x:v>
       </x:c>
       <x:c r="X23" t="str">
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="Y23" s="50" t="n">
-        <x:f>IFERROR(C14/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z23" t="str">
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="AA23" s="50" t="n">
-        <x:f>IFERROR(D14/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.006699620844445446</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0067</x:v>
       </x:c>
       <x:c r="AB23" t="str">
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="AC23" s="50" t="n">
-        <x:f>IFERROR(E14/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.025997995871591892</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.026000000000000002</x:v>
       </x:c>
       <x:c r="AD23" t="str">
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="AE23" s="50" t="n">
-        <x:f>IFERROR(F14/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.008264384263091475</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.010100000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -5094,36 +5094,36 @@
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="W24" s="50" t="n">
-        <x:f>IFERROR(B15/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.19618526402005568</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19620000000000004</x:v>
       </x:c>
       <x:c r="X24" t="str">
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="Y24" s="50" t="n">
-        <x:f>IFERROR(C15/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.15303407086143878</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.153</x:v>
       </x:c>
       <x:c r="Z24" t="str">
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="AA24" s="50" t="n">
-        <x:f>IFERROR(D15/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.04132577223931945</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.041299999999999996</x:v>
       </x:c>
       <x:c r="AB24" t="str">
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="AC24" s="50" t="n">
-        <x:f>IFERROR(E15/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.11348504243312058</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.11349999999999999</x:v>
       </x:c>
       <x:c r="AD24" t="str">
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="AE24" s="50" t="n">
-        <x:f>IFERROR(F15/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.15690244842157178</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.126</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -5154,36 +5154,36 @@
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="W25" s="50" t="n">
-        <x:f>IFERROR(B16/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.09984550447424796</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.09980000000000001</x:v>
       </x:c>
       <x:c r="X25" t="str">
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="Y25" s="50" t="n">
-        <x:f>IFERROR(C16/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.0916799938109248</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0917</x:v>
       </x:c>
       <x:c r="Z25" t="str">
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="AA25" s="50" t="n">
-        <x:f>IFERROR(D16/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.05723078108951537</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.057300000000000004</x:v>
       </x:c>
       <x:c r="AB25" t="str">
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="AC25" s="50" t="n">
-        <x:f>IFERROR(E16/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.04871324519612813</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0487</x:v>
       </x:c>
       <x:c r="AD25" t="str">
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="AE25" s="50" t="n">
-        <x:f>IFERROR(F16/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.08690599441119398</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.07437500000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -5214,36 +5214,36 @@
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="W26" s="50" t="n">
-        <x:f>IFERROR(B17/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.26363949139013715</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.26360000000000006</x:v>
       </x:c>
       <x:c r="X26" t="str">
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="Y26" s="50" t="n">
-        <x:f>IFERROR(C17/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.2029891652515887</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.203</x:v>
       </x:c>
       <x:c r="Z26" t="str">
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="AA26" s="50" t="n">
-        <x:f>IFERROR(D17/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.13581027618122676</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1358</x:v>
       </x:c>
       <x:c r="AB26" t="str">
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="AC26" s="50" t="n">
-        <x:f>IFERROR(E17/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.1919061476786995</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19190000000000002</x:v>
       </x:c>
       <x:c r="AD26" t="str">
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="AE26" s="50" t="n">
-        <x:f>IFERROR(F17/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.22780196583383455</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.198575</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -5274,36 +5274,36 @@
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="W27" s="50" t="n">
-        <x:f>IFERROR(B18/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.09777056332698032</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.09780000000000001</x:v>
       </x:c>
       <x:c r="X27" t="str">
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="Y27" s="50" t="n">
-        <x:f>IFERROR(C18/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.10047580814998996</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1005</x:v>
       </x:c>
       <x:c r="Z27" t="str">
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="AA27" s="50" t="n">
-        <x:f>IFERROR(D18/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.08338056969282108</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0834</x:v>
       </x:c>
       <x:c r="AB27" t="str">
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="AC27" s="50" t="n">
-        <x:f>IFERROR(E18/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.03416657549949762</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0342</x:v>
       </x:c>
       <x:c r="AD27" t="str">
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="AE27" s="50" t="n">
-        <x:f>IFERROR(F18/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.08984998219732857</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.078975</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -5337,7 +5337,7 @@
     <x:mergeCell ref="A3:T3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17f8b8e6b71c4f77"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f6a7ed608974b44"/>
 </x:worksheet>
 </file>
 
@@ -5661,36 +5661,36 @@
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="W12" s="50" t="n">
-        <x:f>IFERROR(B19/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.08591007743801093</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.08010000000000002</x:v>
       </x:c>
       <x:c r="X12" t="str">
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="Y12" s="50" t="n">
-        <x:f>IFERROR(C19/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.11349116086939169</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.2029</x:v>
       </x:c>
       <x:c r="Z12" t="str">
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="AA12" s="50" t="n">
-        <x:f>IFERROR(D19/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.1057019622523328</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0983</x:v>
       </x:c>
       <x:c r="AB12" t="str">
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="AC12" s="50" t="n">
-        <x:f>IFERROR(E19/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.05249307537496133</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.048</x:v>
       </x:c>
       <x:c r="AD12" t="str">
         <x:v>轉存金融機構</x:v>
       </x:c>
       <x:c r="AE12" s="50" t="n">
-        <x:f>IFERROR(F19/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.10253316430655338</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.107325</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -5721,35 +5721,35 @@
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="W13" s="50" t="n">
-        <x:f>IFERROR(B20/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X13" t="str">
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="Y13" s="50" t="n">
-        <x:f>IFERROR(C20/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z13" t="str">
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="AA13" s="50" t="n">
-        <x:f>IFERROR(D20/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB13" t="str">
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="AC13" s="50" t="n">
-        <x:f>IFERROR(E20/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD13" t="str">
         <x:v>政策性貸款</x:v>
       </x:c>
       <x:c r="AE13" s="50" t="n">
-        <x:f>IFERROR(F20/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5781,36 +5781,36 @@
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="W14" s="50" t="n">
-        <x:f>IFERROR(B21/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.025600000000000005</x:v>
       </x:c>
       <x:c r="X14" t="str">
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="Y14" s="50" t="n">
-        <x:f>IFERROR(C21/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.475007680466909</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.061200000000000004</x:v>
       </x:c>
       <x:c r="Z14" t="str">
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="AA14" s="50" t="n">
-        <x:f>IFERROR(D21/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.026099999999999998</x:v>
       </x:c>
       <x:c r="AB14" t="str">
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="AC14" s="50" t="n">
-        <x:f>IFERROR(E21/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0174</x:v>
       </x:c>
       <x:c r="AD14" t="str">
         <x:v>短期票券</x:v>
       </x:c>
       <x:c r="AE14" s="50" t="n">
-        <x:f>IFERROR(F21/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.032575</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -5841,36 +5841,36 @@
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="W15" s="50" t="n">
-        <x:f>IFERROR(B22/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.042100000000000005</x:v>
       </x:c>
       <x:c r="X15" t="str">
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="Y15" s="50" t="n">
-        <x:f>IFERROR(C22/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z15" t="str">
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="AA15" s="50" t="n">
-        <x:f>IFERROR(D22/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.043899999999999995</x:v>
       </x:c>
       <x:c r="AB15" t="str">
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="AC15" s="50" t="n">
-        <x:f>IFERROR(E22/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0691</x:v>
       </x:c>
       <x:c r="AD15" t="str">
         <x:v>公債、公司債、金融債券及特別股</x:v>
       </x:c>
       <x:c r="AE15" s="50" t="n">
-        <x:f>IFERROR(F22/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.038775</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -5901,36 +5901,36 @@
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="W16" s="50" t="n">
-        <x:f>IFERROR(B23/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X16" t="str">
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="Y16" s="50" t="n">
-        <x:f>IFERROR(C23/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.040466652577802666</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0724</x:v>
       </x:c>
       <x:c r="Z16" t="str">
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="AA16" s="50" t="n">
-        <x:f>IFERROR(D23/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB16" t="str">
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="AC16" s="50" t="n">
-        <x:f>IFERROR(E23/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD16" t="str">
         <x:v>公債、金融債券、公司債及證券化商品</x:v>
       </x:c>
       <x:c r="AE16" s="50" t="n">
-        <x:f>IFERROR(F23/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.00961100816252155</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0181</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -5961,36 +5961,36 @@
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="W17" s="50" t="n">
-        <x:f>IFERROR(B24/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X17" t="str">
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="Y17" s="50" t="n">
-        <x:f>IFERROR(C24/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z17" t="str">
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="AA17" s="50" t="n">
-        <x:f>IFERROR(D24/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.0010188259302816812</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0009</x:v>
       </x:c>
       <x:c r="AB17" t="str">
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="AC17" s="50" t="n">
-        <x:f>IFERROR(E24/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD17" t="str">
         <x:v>房屋及土地</x:v>
       </x:c>
       <x:c r="AE17" s="50" t="n">
-        <x:f>IFERROR(F24/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.00017353785290100476</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.000225</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -6021,36 +6021,36 @@
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="W18" s="50" t="n">
-        <x:f>IFERROR(B25/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X18" t="str">
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="Y18" s="50" t="n">
-        <x:f>IFERROR(C25/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z18" t="str">
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="AA18" s="50" t="n">
-        <x:f>IFERROR(D25/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.00048678091810010486</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0005</x:v>
       </x:c>
       <x:c r="AB18" t="str">
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="AC18" s="50" t="n">
-        <x:f>IFERROR(E25/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD18" t="str">
         <x:v>政府或公營事業貸款</x:v>
       </x:c>
       <x:c r="AE18" s="50" t="n">
-        <x:f>IFERROR(F25/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.00008291398250623317</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.000125</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -6081,36 +6081,36 @@
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="W19" s="50" t="n">
-        <x:f>IFERROR(B26/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X19" t="str">
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="Y19" s="50" t="n">
-        <x:f>IFERROR(C26/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z19" t="str">
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="AA19" s="50" t="n">
-        <x:f>IFERROR(D26/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.02204115775027534</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.020499999999999997</x:v>
       </x:c>
       <x:c r="AB19" t="str">
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="AC19" s="50" t="n">
-        <x:f>IFERROR(E26/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD19" t="str">
         <x:v>被保險人貸款</x:v>
       </x:c>
       <x:c r="AE19" s="50" t="n">
-        <x:f>IFERROR(F26/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.0037542970567873246</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.005124999999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -6141,36 +6141,36 @@
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="W20" s="50" t="n">
-        <x:f>IFERROR(B27/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.055961194533538296</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0522</x:v>
       </x:c>
       <x:c r="X20" t="str">
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="Y20" s="50" t="n">
-        <x:f>IFERROR(C27/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.04034712746974965</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0721</x:v>
       </x:c>
       <x:c r="Z20" t="str">
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="AA20" s="50" t="n">
-        <x:f>IFERROR(D27/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.3331317080001063</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.3098</x:v>
       </x:c>
       <x:c r="AB20" t="str">
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="AC20" s="50" t="n">
-        <x:f>IFERROR(E27/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.28681651089402854</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.262</x:v>
       </x:c>
       <x:c r="AD20" t="str">
         <x:v>股票及受益憑證投資（含期貨）</x:v>
       </x:c>
       <x:c r="AE20" s="50" t="n">
-        <x:f>IFERROR(F27/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.12643820937201783</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.174025</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -6196,36 +6196,36 @@
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="W21" s="50" t="n">
-        <x:f>IFERROR(B12/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.12953267317388073</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.12080000000000002</x:v>
       </x:c>
       <x:c r="X21" t="str">
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="Y21" s="50" t="n">
-        <x:f>IFERROR(C12/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.013877837509840278</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0248</x:v>
       </x:c>
       <x:c r="Z21" t="str">
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="AA21" s="50" t="n">
-        <x:f>IFERROR(D12/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.12378380873949746</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1151</x:v>
       </x:c>
       <x:c r="AB21" t="str">
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="AC21" s="50" t="n">
-        <x:f>IFERROR(E12/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.13403073741045154</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.12240000000000001</x:v>
       </x:c>
       <x:c r="AD21" t="str">
         <x:v>自行運用-國外-固定收益</x:v>
       </x:c>
       <x:c r="AE21" s="50" t="n">
-        <x:f>IFERROR(F12/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.11610091308162436</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.095775</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -6256,36 +6256,36 @@
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="W22" s="50" t="n">
-        <x:f>IFERROR(B13/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.015092963877875721</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.014100000000000001</x:v>
       </x:c>
       <x:c r="X22" t="str">
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="Y22" s="50" t="n">
-        <x:f>IFERROR(C13/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.010259022550242067</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0184</x:v>
       </x:c>
       <x:c r="Z22" t="str">
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="AA22" s="50" t="n">
-        <x:f>IFERROR(D13/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.06498542368738083</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0604</x:v>
       </x:c>
       <x:c r="AB22" t="str">
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="AC22" s="50" t="n">
-        <x:f>IFERROR(E13/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.07315031270084386</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0668</x:v>
       </x:c>
       <x:c r="AD22" t="str">
         <x:v>自行運用-國外-權益證券</x:v>
       </x:c>
       <x:c r="AE22" s="50" t="n">
-        <x:f>IFERROR(F13/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.02934192685892919</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.039925</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -6316,36 +6316,36 @@
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="W23" s="50" t="n">
-        <x:f>IFERROR(B14/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.008290945766926794</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.007700000000000001</x:v>
       </x:c>
       <x:c r="X23" t="str">
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="Y23" s="50" t="n">
-        <x:f>IFERROR(C14/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z23" t="str">
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="AA23" s="50" t="n">
-        <x:f>IFERROR(D14/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.0072035334470178895</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0067</x:v>
       </x:c>
       <x:c r="AB23" t="str">
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="AC23" s="50" t="n">
-        <x:f>IFERROR(E14/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.028460576033988435</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.026000000000000002</x:v>
       </x:c>
       <x:c r="AD23" t="str">
         <x:v>自行運用-國外-另類投資</x:v>
       </x:c>
       <x:c r="AE23" s="50" t="n">
-        <x:f>IFERROR(F14/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.008877103672406713</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.010100000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -6376,36 +6376,36 @@
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="W24" s="50" t="n">
-        <x:f>IFERROR(B15/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.2104405841765572</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19620000000000004</x:v>
       </x:c>
       <x:c r="X24" t="str">
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="Y24" s="50" t="n">
-        <x:f>IFERROR(C15/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.08557910923436605</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.153</x:v>
       </x:c>
       <x:c r="Z24" t="str">
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="AA24" s="50" t="n">
-        <x:f>IFERROR(D15/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.044434094027364646</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.041299999999999996</x:v>
       </x:c>
       <x:c r="AB24" t="str">
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="AC24" s="50" t="n">
-        <x:f>IFERROR(E15/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.12423456388103749</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.11349999999999999</x:v>
       </x:c>
       <x:c r="AD24" t="str">
         <x:v>委託經營-國內-權益證券</x:v>
       </x:c>
       <x:c r="AE24" s="50" t="n">
-        <x:f>IFERROR(F15/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.168535157218321</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.126</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -6436,36 +6436,36 @@
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="W25" s="50" t="n">
-        <x:f>IFERROR(B16/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.10710053272306842</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.09980000000000001</x:v>
       </x:c>
       <x:c r="X25" t="str">
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="Y25" s="50" t="n">
-        <x:f>IFERROR(C16/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.05126892436949562</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0917</x:v>
       </x:c>
       <x:c r="Z25" t="str">
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="AA25" s="50" t="n">
-        <x:f>IFERROR(D16/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.061535399591916395</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.057300000000000004</x:v>
       </x:c>
       <x:c r="AB25" t="str">
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="AC25" s="50" t="n">
-        <x:f>IFERROR(E16/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.05332745745535172</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0487</x:v>
       </x:c>
       <x:c r="AD25" t="str">
         <x:v>委託經營-國外-固定收益</x:v>
       </x:c>
       <x:c r="AE25" s="50" t="n">
-        <x:f>IFERROR(F16/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.09334918338528231</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.07437500000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -6496,36 +6496,36 @@
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="W26" s="50" t="n">
-        <x:f>IFERROR(B17/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.28279620723439863</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.26360000000000006</x:v>
       </x:c>
       <x:c r="X26" t="str">
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="Y26" s="50" t="n">
-        <x:f>IFERROR(C17/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.11351479999631743</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.203</x:v>
       </x:c>
       <x:c r="Z26" t="str">
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="AA26" s="50" t="n">
-        <x:f>IFERROR(D17/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.14602525868778218</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1358</x:v>
       </x:c>
       <x:c r="AB26" t="str">
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="AC26" s="50" t="n">
-        <x:f>IFERROR(E17/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.21008386701713133</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19190000000000002</x:v>
       </x:c>
       <x:c r="AD26" t="str">
         <x:v>委託經營-國外-權益證券</x:v>
       </x:c>
       <x:c r="AE26" s="50" t="n">
-        <x:f>IFERROR(F17/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.24469114735095152</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.198575</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -6556,36 +6556,36 @@
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="W27" s="50" t="n">
-        <x:f>IFERROR(B18/SUM(B19,B20,B21,B22,B23,B24,B25,B26,B27,B12,B13,B14,B15,B16,B17,B18),0)</x:f>
-        <x:v>0.10487482107574338</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.09780000000000001</x:v>
       </x:c>
       <x:c r="X27" t="str">
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="Y27" s="50" t="n">
-        <x:f>IFERROR(C18/SUM(C19,C20,C21,C22,C23,C24,C25,C26,C27,C12,C13,C14,C15,C16,C17,C18),0)</x:f>
-        <x:v>0.05618768495588562</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1005</x:v>
       </x:c>
       <x:c r="Z27" t="str">
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="AA27" s="50" t="n">
-        <x:f>IFERROR(D18/SUM(D19,D20,D21,D22,D23,D24,D25,D26,D27,D12,D13,D14,D15,D16,D17,D18),0)</x:f>
-        <x:v>0.08965204696794446</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0834</x:v>
       </x:c>
       <x:c r="AB27" t="str">
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="AC27" s="50" t="n">
-        <x:f>IFERROR(E18/SUM(E19,E20,E21,E22,E23,E24,E25,E26,E27,E12,E13,E14,E15,E16,E17,E18),0)</x:f>
-        <x:v>0.03740289923220597</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0342</x:v>
       </x:c>
       <x:c r="AD27" t="str">
         <x:v>委託經營-國外-另類投資</x:v>
       </x:c>
       <x:c r="AE27" s="50" t="n">
-        <x:f>IFERROR(F18/SUM(F19,F20,F21,F22,F23,F24,F25,F26,F27,F12,F13,F14,F15,F16,F17,F18),0)</x:f>
-        <x:v>0.09651143769919772</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.078975</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -6621,7 +6621,7 @@
     <x:mergeCell ref="A22:F22"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd24b9563f4cd4b65"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68f018aaa4f94ad0"/>
 </x:worksheet>
 </file>
 
@@ -13443,7 +13443,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb66c285481594b01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74e78f0887e1484d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18482,7 +18482,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2577bbb40c2840e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd45515c2be7a4ac8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26461,7 +26461,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5cb1800467847e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cf4438ae6a04441"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30400,7 +30400,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R449830fedb6e4c60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12862eef213a4eae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32564,7 +32564,7 @@
     <x:mergeCell ref="A1:AB1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ecc9d40823948cb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4068634ba3d4894"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Group pie chart residual assets and normalize manager aliases
</commit_message>
<xml_diff>
--- a/outputs/blf-monthly-disclosure/勞工退休基金月度揭露_可持續更新.xlsx
+++ b/outputs/blf-monthly-disclosure/勞工退休基金月度揭露_可持續更新.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板" sheetId="1" r:id="R669daac13ad74f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板(美元)" sheetId="2" r:id="R33a107dc429342d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度資產配置" sheetId="3" r:id="R038d41fa085c48ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國內委外明細" sheetId="4" r:id="R90f8d2ff99c0436a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國外委外明細" sheetId="5" r:id="R98c7add857854f5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次彙總" sheetId="6" r:id="R95dcd709b20e4a79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業者彙總" sheetId="7" r:id="R655147c3abff4a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新說明" sheetId="8" r:id="Rd797195441a049c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料品質檢核" sheetId="9" r:id="R00327db2d15443fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板" sheetId="1" r:id="Rea57131bbd824ffa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板(美元)" sheetId="2" r:id="Rc7f6dd0ef8624f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度資產配置" sheetId="3" r:id="R8f610c8024324425"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國內委外明細" sheetId="4" r:id="R503ecde672d34e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國外委外明細" sheetId="5" r:id="R4ebe21c7b8d64aff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次彙總" sheetId="6" r:id="R802666f003924e1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業者彙總" sheetId="7" r:id="R9c0fb9a211e949db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新說明" sheetId="8" r:id="Red807b104c3e47b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料品質檢核" sheetId="9" r:id="R435746bd90384b4e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,118 +571,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$V$12:$V$27</c:f>
+              <c:f>'儀表板'!$V$12:$V$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -690,7 +582,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$W$12:$W$27</c:f>
+              <c:f>'儀表板'!$W$12:$W$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -781,118 +673,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$AD$12:$AD$27</c:f>
+              <c:f>'儀表板(美元)'!$AD$12:$AD$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -900,7 +684,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$AE$12:$AE$27</c:f>
+              <c:f>'儀表板(美元)'!$AE$12:$AE$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1733,118 +1517,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$X$12:$X$27</c:f>
+              <c:f>'儀表板'!$X$12:$X$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1852,7 +1528,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$Y$12:$Y$27</c:f>
+              <c:f>'儀表板'!$Y$12:$Y$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1943,118 +1619,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$Z$12:$Z$27</c:f>
+              <c:f>'儀表板'!$Z$12:$Z$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -2062,7 +1630,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$AA$12:$AA$27</c:f>
+              <c:f>'儀表板'!$AA$12:$AA$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -2153,118 +1721,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$AB$12:$AB$27</c:f>
+              <c:f>'儀表板'!$AB$12:$AB$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -2272,7 +1732,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$AC$12:$AC$27</c:f>
+              <c:f>'儀表板'!$AC$12:$AC$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -2363,118 +1823,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$AD$12:$AD$27</c:f>
+              <c:f>'儀表板'!$AD$12:$AD$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -2482,7 +1834,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$AE$12:$AE$27</c:f>
+              <c:f>'儀表板'!$AE$12:$AE$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -2573,118 +1925,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$V$12:$V$27</c:f>
+              <c:f>'儀表板(美元)'!$V$12:$V$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -2692,7 +1936,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$W$12:$W$27</c:f>
+              <c:f>'儀表板(美元)'!$W$12:$W$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -2783,118 +2027,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$X$12:$X$27</c:f>
+              <c:f>'儀表板(美元)'!$X$12:$X$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -2902,7 +2038,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$Y$12:$Y$27</c:f>
+              <c:f>'儀表板(美元)'!$Y$12:$Y$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -2993,118 +2129,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$Z$12:$Z$27</c:f>
+              <c:f>'儀表板(美元)'!$Z$12:$Z$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -3112,7 +2140,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$AA$12:$AA$27</c:f>
+              <c:f>'儀表板(美元)'!$AA$12:$AA$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -3203,118 +2231,10 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="4"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="5"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="6"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="8"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="9"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="10"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="11"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="12"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="13"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="14"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="15"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$AB$12:$AB$27</c:f>
+              <c:f>'儀表板(美元)'!$AB$12:$AB$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -3322,7 +2242,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$AC$12:$AC$27</c:f>
+              <c:f>'儀表板(美元)'!$AC$12:$AC$15</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -3375,7 +2295,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8bcbffc68bdd42c7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rddc8e118ed474418"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3405,7 +2325,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re347ddf758a443cf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6b65fbf37bde4894"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3435,7 +2355,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8327dbd615e5436d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a329b0c78c647c2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3465,7 +2385,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc802eff804884510"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b4a3c4fd0d84121"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3495,7 +2415,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra942c1960ef0439b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R55ef10ffbb394b03"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3530,7 +2450,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ref3eb68545f84288"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb2a6c0d367bd46fa"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3560,7 +2480,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R06365c72ff574aa6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R56c9937843464ec6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3590,7 +2510,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8fabfa9601cf43b8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1c39af05f56c4eb8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3620,7 +2540,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3b8271fb31fc4e07"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra0ea1935afa845af"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3650,7 +2570,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9e842dc2cb7e4bfb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbe4c7fa4cb2f4027"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3685,7 +2605,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc1c31b906090403b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca4d8f8b1ada4398"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3715,7 +2635,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R73cbe4e5c09a4c57"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R19e78b81399f4313"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3745,7 +2665,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Reda42996294f4f1d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc4beec4e9e464d05"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3775,7 +2695,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3ca6cd30a901413c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfce1f130435241f8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4192,7 +3112,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="J6" s="58" t="n">
-        <x:v>50</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="K6" s="59" t="str">
         <x:v>詳見「業者彙總」</x:v>
@@ -4371,39 +3291,39 @@
         <x:v>來源與報價時間已註明</x:v>
       </x:c>
       <x:c r="V12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="W12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.08010000000000002</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.22060000000000002</x:v>
       </x:c>
       <x:c r="X12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="Y12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.2029</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1165</x:v>
       </x:c>
       <x:c r="Z12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="AA12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0983</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1724</x:v>
       </x:c>
       <x:c r="AB12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="AC12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.048</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1711</x:v>
       </x:c>
       <x:c r="AD12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="AE12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.107325</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.45747499999999997</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4431,39 +3351,39 @@
         <x:v>2654.12955439</x:v>
       </x:c>
       <x:c r="V13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="W13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.4739</x:v>
       </x:c>
       <x:c r="X13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="Y13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.3744</x:v>
       </x:c>
       <x:c r="Z13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="AA13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.2375</x:v>
       </x:c>
       <x:c r="AB13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="AC13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.3722</x:v>
       </x:c>
       <x:c r="AD13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="AE13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.8622749999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4491,39 +3411,39 @@
         <x:v>802.98009492</x:v>
       </x:c>
       <x:c r="V14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="W14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.025600000000000005</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1055</x:v>
       </x:c>
       <x:c r="X14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="Y14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.061200000000000004</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1005</x:v>
       </x:c>
       <x:c r="Z14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="AA14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.026099999999999998</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.0901</x:v>
       </x:c>
       <x:c r="AB14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="AC14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0174</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.060200000000000004</x:v>
       </x:c>
       <x:c r="AD14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="AE14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.032575</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.119375</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -4551,39 +3471,39 @@
         <x:v>15244.879584</x:v>
       </x:c>
       <x:c r="V15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="W15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.042100000000000005</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.19999999999999998</x:v>
       </x:c>
       <x:c r="X15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="Y15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.4086</x:v>
       </x:c>
       <x:c r="Z15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="AA15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.043899999999999995</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="AB15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="AC15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0691</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.3965</x:v>
       </x:c>
       <x:c r="AD15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="AE15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.038775</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.9830249999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -4610,41 +3530,6 @@
         <x:f>SUM(B16:E16)</x:f>
         <x:v>8443.91807301</x:v>
       </x:c>
-      <x:c r="V16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="W16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="X16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="Y16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0724</x:v>
-      </x:c>
-      <x:c r="Z16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="AA16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AB16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="AC16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="AE16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0181</x:v>
-      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="30" t="str">
@@ -4670,41 +3555,6 @@
         <x:f>SUM(B17:E17)</x:f>
         <x:v>22133.584103189998</x:v>
       </x:c>
-      <x:c r="V17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="W17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="X17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="Y17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Z17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="AA17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0009</x:v>
-      </x:c>
-      <x:c r="AB17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="AC17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="AE17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.000225</x:v>
-      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="30" t="str">
@@ -4730,41 +3580,6 @@
         <x:f>SUM(B18:E18)</x:f>
         <x:v>8729.960386230001</x:v>
       </x:c>
-      <x:c r="V18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="W18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="X18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="Y18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Z18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="AA18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0005</x:v>
-      </x:c>
-      <x:c r="AB18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="AC18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="AE18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.000125</x:v>
-      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="30" t="str">
@@ -4790,41 +3605,6 @@
         <x:f>SUM(B19:E19)</x:f>
         <x:v>9274.65680763</x:v>
       </x:c>
-      <x:c r="V19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="W19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="X19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="Y19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Z19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="AA19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.020499999999999997</x:v>
-      </x:c>
-      <x:c r="AB19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="AC19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="AE19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.005124999999999999</x:v>
-      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="30" t="str">
@@ -4850,41 +3630,6 @@
         <x:f>SUM(B20:E20)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="V20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="W20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0522</x:v>
-      </x:c>
-      <x:c r="X20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="Y20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0721</x:v>
-      </x:c>
-      <x:c r="Z20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="AA20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.3098</x:v>
-      </x:c>
-      <x:c r="AB20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="AC20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.262</x:v>
-      </x:c>
-      <x:c r="AD20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="AE20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.174025</x:v>
-      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="30" t="str">
@@ -4910,41 +3655,6 @@
         <x:f>SUM(B21:E21)</x:f>
         <x:v>2849.5867313800004</x:v>
       </x:c>
-      <x:c r="V21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="W21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.12080000000000002</x:v>
-      </x:c>
-      <x:c r="X21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="Y21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0248</x:v>
-      </x:c>
-      <x:c r="Z21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AA21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.1151</x:v>
-      </x:c>
-      <x:c r="AB21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AC21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.12240000000000001</x:v>
-      </x:c>
-      <x:c r="AD21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AE21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.095775</x:v>
-      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="30" t="str">
@@ -4970,41 +3680,6 @@
         <x:f>SUM(B22:E22)</x:f>
         <x:v>3856.7386907</x:v>
       </x:c>
-      <x:c r="V22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="W22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.014100000000000001</x:v>
-      </x:c>
-      <x:c r="X22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="Y22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0184</x:v>
-      </x:c>
-      <x:c r="Z22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AA22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0604</x:v>
-      </x:c>
-      <x:c r="AB22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AC22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0668</x:v>
-      </x:c>
-      <x:c r="AD22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AE22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.039925</x:v>
-      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="30" t="str">
@@ -5030,41 +3705,6 @@
         <x:f>SUM(B23:E23)</x:f>
         <x:v>869.36556465</x:v>
       </x:c>
-      <x:c r="V23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="W23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.007700000000000001</x:v>
-      </x:c>
-      <x:c r="X23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="Y23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Z23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AA23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0067</x:v>
-      </x:c>
-      <x:c r="AB23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AC23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.026000000000000002</x:v>
-      </x:c>
-      <x:c r="AD23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AE23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.010100000000000001</x:v>
-      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="30" t="str">
@@ -5090,41 +3730,6 @@
         <x:f>SUM(B24:E24)</x:f>
         <x:v>15.69739937</x:v>
       </x:c>
-      <x:c r="V24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="W24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.19620000000000004</x:v>
-      </x:c>
-      <x:c r="X24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="Y24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.153</x:v>
-      </x:c>
-      <x:c r="Z24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="AA24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.041299999999999996</x:v>
-      </x:c>
-      <x:c r="AB24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="AC24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.11349999999999999</x:v>
-      </x:c>
-      <x:c r="AD24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="AE24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.126</x:v>
-      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="30" t="str">
@@ -5150,41 +3755,6 @@
         <x:f>SUM(B25:E25)</x:f>
         <x:v>7.5</x:v>
       </x:c>
-      <x:c r="V25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="W25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.09980000000000001</x:v>
-      </x:c>
-      <x:c r="X25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="Y25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0917</x:v>
-      </x:c>
-      <x:c r="Z25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AA25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.057300000000000004</x:v>
-      </x:c>
-      <x:c r="AB25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AC25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0487</x:v>
-      </x:c>
-      <x:c r="AD25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AE25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.07437500000000001</x:v>
-      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="30" t="str">
@@ -5210,41 +3780,6 @@
         <x:f>SUM(B26:E26)</x:f>
         <x:v>339.59565172</x:v>
       </x:c>
-      <x:c r="V26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="W26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.26360000000000006</x:v>
-      </x:c>
-      <x:c r="X26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="Y26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.203</x:v>
-      </x:c>
-      <x:c r="Z26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AA26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.1358</x:v>
-      </x:c>
-      <x:c r="AB26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AC26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.19190000000000002</x:v>
-      </x:c>
-      <x:c r="AD26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AE26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.198575</x:v>
-      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="30" t="str">
@@ -5269,41 +3804,6 @@
       <x:c r="F27" s="66" t="n">
         <x:f>SUM(B27:E27)</x:f>
         <x:v>11436.992189089999</x:v>
-      </x:c>
-      <x:c r="V27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="W27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.09780000000000001</x:v>
-      </x:c>
-      <x:c r="X27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="Y27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.1005</x:v>
-      </x:c>
-      <x:c r="Z27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AA27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0834</x:v>
-      </x:c>
-      <x:c r="AB27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AC27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0342</x:v>
-      </x:c>
-      <x:c r="AD27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AE27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.078975</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -5337,7 +3837,7 @@
     <x:mergeCell ref="A3:T3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f6a7ed608974b44"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e123d448f714b76"/>
 </x:worksheet>
 </file>
 
@@ -5479,7 +3979,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="J6" s="58" t="n">
-        <x:v>50</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="K6" s="59" t="str">
         <x:v>詳見「業者彙總」</x:v>
@@ -5658,39 +4158,39 @@
         <x:v>來源與報價時間已註明</x:v>
       </x:c>
       <x:c r="V12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="W12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.08010000000000002</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.22060000000000002</x:v>
       </x:c>
       <x:c r="X12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="Y12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.2029</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1165</x:v>
       </x:c>
       <x:c r="Z12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="AA12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0983</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1724</x:v>
       </x:c>
       <x:c r="AB12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="AC12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.048</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1711</x:v>
       </x:c>
       <x:c r="AD12" t="str">
-        <x:v>轉存金融機構</x:v>
+        <x:v>固定收益</x:v>
       </x:c>
       <x:c r="AE12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.107325</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.45747499999999997</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -5718,39 +4218,39 @@
         <x:v>8.30843498009078</x:v>
       </x:c>
       <x:c r="V13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="W13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.4739</x:v>
       </x:c>
       <x:c r="X13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="Y13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.3744</x:v>
       </x:c>
       <x:c r="Z13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="AA13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.2375</x:v>
       </x:c>
       <x:c r="AB13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="AC13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.3722</x:v>
       </x:c>
       <x:c r="AD13" t="str">
-        <x:v>政策性貸款</x:v>
+        <x:v>權益證券</x:v>
       </x:c>
       <x:c r="AE13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.8622749999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -5778,39 +4278,39 @@
         <x:v>2.513633103521678</x:v>
       </x:c>
       <x:c r="V14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="W14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.025600000000000005</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1055</x:v>
       </x:c>
       <x:c r="X14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="Y14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.061200000000000004</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.1005</x:v>
       </x:c>
       <x:c r="Z14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="AA14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.026099999999999998</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.0901</x:v>
       </x:c>
       <x:c r="AB14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="AC14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0174</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.060200000000000004</x:v>
       </x:c>
       <x:c r="AD14" t="str">
-        <x:v>短期票券</x:v>
+        <x:v>另類投資</x:v>
       </x:c>
       <x:c r="AE14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.032575</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.119375</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -5838,39 +4338,39 @@
         <x:v>47.7222713538895</x:v>
       </x:c>
       <x:c r="V15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="W15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.042100000000000005</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.19999999999999998</x:v>
       </x:c>
       <x:c r="X15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="Y15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.4086</x:v>
       </x:c>
       <x:c r="Z15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="AA15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.043899999999999995</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="AB15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="AC15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0691</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.3965</x:v>
       </x:c>
       <x:c r="AD15" t="str">
-        <x:v>公債、公司債、金融債券及特別股</x:v>
+        <x:v>其他</x:v>
       </x:c>
       <x:c r="AE15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.038775</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
+        <x:v>0.9830249999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -5897,41 +4397,6 @@
         <x:f>SUM(B16:E16)</x:f>
         <x:v>26.432675138550632</x:v>
       </x:c>
-      <x:c r="V16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="W16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="X16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="Y16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0724</x:v>
-      </x:c>
-      <x:c r="Z16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="AA16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AB16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="AC16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD16" t="str">
-        <x:v>公債、金融債券、公司債及證券化商品</x:v>
-      </x:c>
-      <x:c r="AE16" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0181</x:v>
-      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="30" t="str">
@@ -5957,41 +4422,6 @@
         <x:f>SUM(B17:E17)</x:f>
         <x:v>69.28653655717639</x:v>
       </x:c>
-      <x:c r="V17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="W17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="X17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="Y17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Z17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="AA17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0009</x:v>
-      </x:c>
-      <x:c r="AB17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="AC17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD17" t="str">
-        <x:v>房屋及土地</x:v>
-      </x:c>
-      <x:c r="AE17" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.000225</x:v>
-      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="30" t="str">
@@ -6017,41 +4447,6 @@
         <x:f>SUM(B18:E18)</x:f>
         <x:v>27.32809637260917</x:v>
       </x:c>
-      <x:c r="V18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="W18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="X18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="Y18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Z18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="AA18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0005</x:v>
-      </x:c>
-      <x:c r="AB18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="AC18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD18" t="str">
-        <x:v>政府或公營事業貸款</x:v>
-      </x:c>
-      <x:c r="AE18" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.000125</x:v>
-      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="30" t="str">
@@ -6077,41 +4472,6 @@
         <x:f>SUM(B19:E19)</x:f>
         <x:v>29.033203342087965</x:v>
       </x:c>
-      <x:c r="V19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="W19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="X19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="Y19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Z19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="AA19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.020499999999999997</x:v>
-      </x:c>
-      <x:c r="AB19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="AC19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD19" t="str">
-        <x:v>被保險人貸款</x:v>
-      </x:c>
-      <x:c r="AE19" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.005124999999999999</x:v>
-      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="81" t="str">
@@ -6137,41 +4497,6 @@
         <x:f>SUM(B20:E20)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="V20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="W20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0522</x:v>
-      </x:c>
-      <x:c r="X20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="Y20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0721</x:v>
-      </x:c>
-      <x:c r="Z20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="AA20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.3098</x:v>
-      </x:c>
-      <x:c r="AB20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="AC20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.262</x:v>
-      </x:c>
-      <x:c r="AD20" t="str">
-        <x:v>股票及受益憑證投資（含期貨）</x:v>
-      </x:c>
-      <x:c r="AE20" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.174025</x:v>
-      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="30" t="str">
@@ -6192,41 +4517,6 @@
       <x:c r="F21" s="74" t="str">
         <x:v>TWD／USD</x:v>
       </x:c>
-      <x:c r="V21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="W21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.12080000000000002</x:v>
-      </x:c>
-      <x:c r="X21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="Y21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0248</x:v>
-      </x:c>
-      <x:c r="Z21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AA21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.1151</x:v>
-      </x:c>
-      <x:c r="AB21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AC21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.12240000000000001</x:v>
-      </x:c>
-      <x:c r="AD21" t="str">
-        <x:v>自行運用-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AE21" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.095775</x:v>
-      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="90" t="str">
@@ -6252,41 +4542,6 @@
         <x:f>SUM(B22:E22)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="V22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="W22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.014100000000000001</x:v>
-      </x:c>
-      <x:c r="X22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="Y22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0184</x:v>
-      </x:c>
-      <x:c r="Z22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AA22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0604</x:v>
-      </x:c>
-      <x:c r="AB22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AC22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0668</x:v>
-      </x:c>
-      <x:c r="AD22" t="str">
-        <x:v>自行運用-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AE22" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.039925</x:v>
-      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="30" t="str">
@@ -6312,41 +4567,6 @@
         <x:f>SUM(B23:E23)</x:f>
         <x:v>2.721444872906558</x:v>
       </x:c>
-      <x:c r="V23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="W23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.007700000000000001</x:v>
-      </x:c>
-      <x:c r="X23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="Y23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Z23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AA23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0067</x:v>
-      </x:c>
-      <x:c r="AB23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AC23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.026000000000000002</x:v>
-      </x:c>
-      <x:c r="AD23" t="str">
-        <x:v>自行運用-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AE23" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.010100000000000001</x:v>
-      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="30" t="str">
@@ -6372,41 +4592,6 @@
         <x:f>SUM(B24:E24)</x:f>
         <x:v>0.049138830395993115</x:v>
       </x:c>
-      <x:c r="V24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="W24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.19620000000000004</x:v>
-      </x:c>
-      <x:c r="X24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="Y24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.153</x:v>
-      </x:c>
-      <x:c r="Z24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="AA24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.041299999999999996</x:v>
-      </x:c>
-      <x:c r="AB24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="AC24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.11349999999999999</x:v>
-      </x:c>
-      <x:c r="AD24" t="str">
-        <x:v>委託經營-國內-權益證券</x:v>
-      </x:c>
-      <x:c r="AE24" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.126</x:v>
-      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="30" t="str">
@@ -6432,41 +4617,6 @@
         <x:f>SUM(B25:E25)</x:f>
         <x:v>0.023477852559085927</x:v>
       </x:c>
-      <x:c r="V25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="W25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.09980000000000001</x:v>
-      </x:c>
-      <x:c r="X25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="Y25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0917</x:v>
-      </x:c>
-      <x:c r="Z25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AA25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.057300000000000004</x:v>
-      </x:c>
-      <x:c r="AB25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AC25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0487</x:v>
-      </x:c>
-      <x:c r="AD25" t="str">
-        <x:v>委託經營-國外-固定收益</x:v>
-      </x:c>
-      <x:c r="AE25" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.07437500000000001</x:v>
-      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="30" t="str">
@@ -6492,41 +4642,6 @@
         <x:f>SUM(B26:E26)</x:f>
         <x:v>1.0630635521051808</x:v>
       </x:c>
-      <x:c r="V26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="W26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.26360000000000006</x:v>
-      </x:c>
-      <x:c r="X26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="Y26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.203</x:v>
-      </x:c>
-      <x:c r="Z26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AA26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.1358</x:v>
-      </x:c>
-      <x:c r="AB26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AC26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.19190000000000002</x:v>
-      </x:c>
-      <x:c r="AD26" t="str">
-        <x:v>委託經營-國外-權益證券</x:v>
-      </x:c>
-      <x:c r="AE26" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.198575</x:v>
-      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="30" t="str">
@@ -6551,41 +4666,6 @@
       <x:c r="F27" s="75" t="n">
         <x:f>SUM(B27:E27)</x:f>
         <x:v>35.80213551131632</x:v>
-      </x:c>
-      <x:c r="V27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="W27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.09780000000000001</x:v>
-      </x:c>
-      <x:c r="X27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="Y27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.1005</x:v>
-      </x:c>
-      <x:c r="Z27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AA27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0834</x:v>
-      </x:c>
-      <x:c r="AB27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AC27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.0342</x:v>
-      </x:c>
-      <x:c r="AD27" t="str">
-        <x:v>委託經營-國外-另類投資</x:v>
-      </x:c>
-      <x:c r="AE27" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
-        <x:v>0.078975</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -6621,7 +4701,7 @@
     <x:mergeCell ref="A22:F22"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68f018aaa4f94ad0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R576dfdfedbb3494b"/>
 </x:worksheet>
 </file>
 
@@ -13443,7 +11523,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74e78f0887e1484d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55ff615b097e473d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18482,7 +16562,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd45515c2be7a4ac8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e109314e2a44d04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22194,7 +20274,7 @@
         <x:v>100-1全球基本面指數被動股票型(續約3)</x:v>
       </x:c>
       <x:c r="F87" s="31" t="str">
-        <x:v>瑞銀</x:v>
+        <x:v>UBS</x:v>
       </x:c>
       <x:c r="G87" s="40" t="n">
         <x:v>361201485</x:v>
@@ -23758,7 +21838,7 @@
         <x:v>104-2全球不動產有價證券型(續約2)</x:v>
       </x:c>
       <x:c r="F123" s="31" t="str">
-        <x:v>信安環球</x:v>
+        <x:v>信安</x:v>
       </x:c>
       <x:c r="G123" s="40" t="n">
         <x:v>425091462</x:v>
@@ -25940,7 +24020,7 @@
         <x:v>100-1全球基本面指數被動股票型(續約2)</x:v>
       </x:c>
       <x:c r="F175" s="31" t="str">
-        <x:v>瑞銀</x:v>
+        <x:v>UBS</x:v>
       </x:c>
       <x:c r="G175" s="40" t="n">
         <x:v>0</x:v>
@@ -26168,7 +24248,7 @@
         <x:v>109年第二次委託經營(相對報酬)</x:v>
       </x:c>
       <x:c r="F181" s="31" t="str">
-        <x:v>安聯</x:v>
+        <x:v>Allianz</x:v>
       </x:c>
       <x:c r="G181" s="40" t="n">
         <x:v>0</x:v>
@@ -26244,7 +24324,7 @@
         <x:v>109年第二次委託經營(相對報酬)</x:v>
       </x:c>
       <x:c r="F183" s="31" t="str">
-        <x:v>野村</x:v>
+        <x:v>Nomura</x:v>
       </x:c>
       <x:c r="G183" s="40" t="n">
         <x:v>0</x:v>
@@ -26461,7 +24541,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cf4438ae6a04441"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6614b9a4d8354037"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30400,7 +28480,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12862eef213a4eae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R234131b6140b42c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30752,11 +28832,11 @@
         <x:v>17827431853</x:v>
       </x:c>
       <x:c r="J9" s="42" t="n">
-        <x:f>IFERROR(I9/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I9/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.1425863938130672</x:v>
       </x:c>
       <x:c r="K9" s="28" t="n">
-        <x:f>RANK(I9,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I9,$I$9:$I$54,0)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="L9" s="29" t="n">
@@ -30830,11 +28910,11 @@
         <x:v>12270337973</x:v>
       </x:c>
       <x:c r="J10" s="43" t="n">
-        <x:f>IFERROR(I10/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I10/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.09813994841568788</x:v>
       </x:c>
       <x:c r="K10" s="31" t="n">
-        <x:f>RANK(I10,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I10,$I$9:$I$54,0)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="L10" s="32" t="n">
@@ -30908,11 +28988,11 @@
         <x:v>8229076099</x:v>
       </x:c>
       <x:c r="J11" s="43" t="n">
-        <x:f>IFERROR(I11/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I11/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.0658173479525746</x:v>
       </x:c>
       <x:c r="K11" s="31" t="n">
-        <x:f>RANK(I11,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I11,$I$9:$I$54,0)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="L11" s="32" t="n">
@@ -30986,11 +29066,11 @@
         <x:v>6499168753</x:v>
       </x:c>
       <x:c r="J12" s="43" t="n">
-        <x:f>IFERROR(I12/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I12/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.05198129730148962</x:v>
       </x:c>
       <x:c r="K12" s="31" t="n">
-        <x:f>RANK(I12,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I12,$I$9:$I$54,0)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="L12" s="32" t="n">
@@ -31064,11 +29144,11 @@
         <x:v>6233333079</x:v>
       </x:c>
       <x:c r="J13" s="43" t="n">
-        <x:f>IFERROR(I13/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I13/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.04985510490232206</x:v>
       </x:c>
       <x:c r="K13" s="31" t="n">
-        <x:f>RANK(I13,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I13,$I$9:$I$54,0)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="L13" s="32" t="n">
@@ -31142,11 +29222,11 @@
         <x:v>5911641695</x:v>
       </x:c>
       <x:c r="J14" s="43" t="n">
-        <x:f>IFERROR(I14/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I14/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.04728217040768952</x:v>
       </x:c>
       <x:c r="K14" s="31" t="n">
-        <x:f>RANK(I14,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I14,$I$9:$I$54,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="L14" s="32" t="n">
@@ -31159,7 +29239,7 @@
         <x:v>其他</x:v>
       </x:c>
       <x:c r="Q14" s="51" t="n">
-        <x:f>SUM(I19:I58)</x:f>
+        <x:f>SUM(I19:I54)</x:f>
         <x:v>49028845422</x:v>
       </x:c>
       <x:c r="R14" s="50" t="n">
@@ -31219,11 +29299,11 @@
         <x:v>5214617387</x:v>
       </x:c>
       <x:c r="J15" s="43" t="n">
-        <x:f>IFERROR(I15/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I15/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.041707268576776396</x:v>
       </x:c>
       <x:c r="K15" s="31" t="n">
-        <x:f>RANK(I15,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I15,$I$9:$I$54,0)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="L15" s="32" t="n">
@@ -31267,11 +29347,11 @@
         <x:v>4884050215</x:v>
       </x:c>
       <x:c r="J16" s="43" t="n">
-        <x:f>IFERROR(I16/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I16/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.0390633442383119</x:v>
       </x:c>
       <x:c r="K16" s="31" t="n">
-        <x:f>RANK(I16,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I16,$I$9:$I$54,0)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="L16" s="32" t="n">
@@ -31315,11 +29395,11 @@
         <x:v>4847721016</x:v>
       </x:c>
       <x:c r="J17" s="43" t="n">
-        <x:f>IFERROR(I17/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I17/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.03877277801889003</x:v>
       </x:c>
       <x:c r="K17" s="31" t="n">
-        <x:f>RANK(I17,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I17,$I$9:$I$54,0)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="L17" s="32" t="n">
@@ -31363,11 +29443,11 @@
         <x:v>4082759823</x:v>
       </x:c>
       <x:c r="J18" s="43" t="n">
-        <x:f>IFERROR(I18/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I18/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.03265450709707709</x:v>
       </x:c>
       <x:c r="K18" s="31" t="n">
-        <x:f>RANK(I18,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I18,$I$9:$I$54,0)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="L18" s="32" t="n">
@@ -31411,11 +29491,11 @@
         <x:v>3525432785</x:v>
       </x:c>
       <x:c r="J19" s="43" t="n">
-        <x:f>IFERROR(I19/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I19/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.028196924357274576</x:v>
       </x:c>
       <x:c r="K19" s="31" t="n">
-        <x:f>RANK(I19,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I19,$I$9:$I$54,0)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="L19" s="32" t="n">
@@ -31459,11 +29539,11 @@
         <x:v>3467884297</x:v>
       </x:c>
       <x:c r="J20" s="43" t="n">
-        <x:f>IFERROR(I20/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I20/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.02773664317707005</x:v>
       </x:c>
       <x:c r="K20" s="31" t="n">
-        <x:f>RANK(I20,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I20,$I$9:$I$54,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="L20" s="32" t="n">
@@ -31507,11 +29587,11 @@
         <x:v>3039287910</x:v>
       </x:c>
       <x:c r="J21" s="43" t="n">
-        <x:f>IFERROR(I21/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I21/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.024308666913996812</x:v>
       </x:c>
       <x:c r="K21" s="31" t="n">
-        <x:f>RANK(I21,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I21,$I$9:$I$54,0)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="L21" s="32" t="n">
@@ -31555,11 +29635,11 @@
         <x:v>3033228329</x:v>
       </x:c>
       <x:c r="J22" s="43" t="n">
-        <x:f>IFERROR(I22/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I22/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.024260201503502884</x:v>
       </x:c>
       <x:c r="K22" s="31" t="n">
-        <x:f>RANK(I22,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I22,$I$9:$I$54,0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="L22" s="32" t="n">
@@ -31603,11 +29683,11 @@
         <x:v>2941839542</x:v>
       </x:c>
       <x:c r="J23" s="43" t="n">
-        <x:f>IFERROR(I23/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I23/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.023529260688206054</x:v>
       </x:c>
       <x:c r="K23" s="31" t="n">
-        <x:f>RANK(I23,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I23,$I$9:$I$54,0)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="L23" s="32" t="n">
@@ -31651,11 +29731,11 @@
         <x:v>2584189383</x:v>
       </x:c>
       <x:c r="J24" s="43" t="n">
-        <x:f>IFERROR(I24/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I24/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.02066872267919953</x:v>
       </x:c>
       <x:c r="K24" s="31" t="n">
-        <x:f>RANK(I24,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I24,$I$9:$I$54,0)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="L24" s="32" t="n">
@@ -31699,11 +29779,11 @@
         <x:v>2458832253</x:v>
       </x:c>
       <x:c r="J25" s="43" t="n">
-        <x:f>IFERROR(I25/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I25/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.019666098114268265</x:v>
       </x:c>
       <x:c r="K25" s="31" t="n">
-        <x:f>RANK(I25,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I25,$I$9:$I$54,0)</x:f>
         <x:v>17</x:v>
       </x:c>
       <x:c r="L25" s="32" t="n">
@@ -31747,11 +29827,11 @@
         <x:v>2389413786</x:v>
       </x:c>
       <x:c r="J26" s="43" t="n">
-        <x:f>IFERROR(I26/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I26/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.019110879114965472</x:v>
       </x:c>
       <x:c r="K26" s="31" t="n">
-        <x:f>RANK(I26,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I26,$I$9:$I$54,0)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="L26" s="32" t="n">
@@ -31772,11 +29852,11 @@
         <x:v>1806278590</x:v>
       </x:c>
       <x:c r="J27" s="43" t="n">
-        <x:f>IFERROR(I27/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I27/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.014446878972447797</x:v>
       </x:c>
       <x:c r="K27" s="31" t="n">
-        <x:f>RANK(I27,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I27,$I$9:$I$54,0)</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="L27" s="32" t="n">
@@ -31797,11 +29877,11 @@
         <x:v>1719232558</x:v>
       </x:c>
       <x:c r="J28" s="43" t="n">
-        <x:f>IFERROR(I28/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I28/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.013750672143502425</x:v>
       </x:c>
       <x:c r="K28" s="31" t="n">
-        <x:f>RANK(I28,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I28,$I$9:$I$54,0)</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="L28" s="32" t="n">
@@ -31822,11 +29902,11 @@
         <x:v>1709168484</x:v>
       </x:c>
       <x:c r="J29" s="43" t="n">
-        <x:f>IFERROR(I29/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I29/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.013670178215349427</x:v>
       </x:c>
       <x:c r="K29" s="31" t="n">
-        <x:f>RANK(I29,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I29,$I$9:$I$54,0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="L29" s="32" t="n">
@@ -31847,11 +29927,11 @@
         <x:v>1679948361</x:v>
       </x:c>
       <x:c r="J30" s="43" t="n">
-        <x:f>IFERROR(I30/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I30/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.013436471420130734</x:v>
       </x:c>
       <x:c r="K30" s="31" t="n">
-        <x:f>RANK(I30,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I30,$I$9:$I$54,0)</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="L30" s="32" t="n">
@@ -31872,11 +29952,11 @@
         <x:v>1388520134</x:v>
       </x:c>
       <x:c r="J31" s="43" t="n">
-        <x:f>IFERROR(I31/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I31/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.011105586058408076</x:v>
       </x:c>
       <x:c r="K31" s="31" t="n">
-        <x:f>RANK(I31,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I31,$I$9:$I$54,0)</x:f>
         <x:v>23</x:v>
       </x:c>
       <x:c r="L31" s="32" t="n">
@@ -31897,11 +29977,11 @@
         <x:v>1352096519</x:v>
       </x:c>
       <x:c r="J32" s="43" t="n">
-        <x:f>IFERROR(I32/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I32/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.01081426468608088</x:v>
       </x:c>
       <x:c r="K32" s="31" t="n">
-        <x:f>RANK(I32,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I32,$I$9:$I$54,0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="L32" s="32" t="n">
@@ -31922,11 +30002,11 @@
         <x:v>1337309953</x:v>
       </x:c>
       <x:c r="J33" s="43" t="n">
-        <x:f>IFERROR(I33/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I33/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.01069599957979951</x:v>
       </x:c>
       <x:c r="K33" s="31" t="n">
-        <x:f>RANK(I33,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I33,$I$9:$I$54,0)</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="L33" s="32" t="n">
@@ -31936,22 +30016,22 @@
     </x:row>
     <x:row r="34">
       <x:c r="G34" s="30" t="str">
-        <x:v>Insight</x:v>
+        <x:v>信安</x:v>
       </x:c>
       <x:c r="H34" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G34,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>1229834121</x:v>
+        <x:v>1133980105</x:v>
       </x:c>
       <x:c r="I34" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G34,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>1218224544</x:v>
+        <x:v>1279212590</x:v>
       </x:c>
       <x:c r="J34" s="43" t="n">
-        <x:f>IFERROR(I34/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.009743537151948088</x:v>
+        <x:f>IFERROR(I34/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.01023132841748486</x:v>
       </x:c>
       <x:c r="K34" s="31" t="n">
-        <x:f>RANK(I34,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I34,$I$9:$I$54,0)</x:f>
         <x:v>26</x:v>
       </x:c>
       <x:c r="L34" s="32" t="n">
@@ -31961,97 +30041,97 @@
     </x:row>
     <x:row r="35">
       <x:c r="G35" s="30" t="str">
-        <x:v>American Century</x:v>
+        <x:v>Insight</x:v>
       </x:c>
       <x:c r="H35" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G35,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>959838014</x:v>
+        <x:v>1229834121</x:v>
       </x:c>
       <x:c r="I35" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G35,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>1175399124</x:v>
+        <x:v>1218224544</x:v>
       </x:c>
       <x:c r="J35" s="43" t="n">
-        <x:f>IFERROR(I35/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.00940101321178211</x:v>
+        <x:f>IFERROR(I35/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.009743537151948088</x:v>
       </x:c>
       <x:c r="K35" s="31" t="n">
-        <x:f>RANK(I35,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I35,$I$9:$I$54,0)</x:f>
         <x:v>27</x:v>
       </x:c>
       <x:c r="L35" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G35,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="G36" s="30" t="str">
-        <x:v>T. Rowe Price</x:v>
+        <x:v>American Century</x:v>
       </x:c>
       <x:c r="H36" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G36,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>960000000</x:v>
+        <x:v>959838014</x:v>
       </x:c>
       <x:c r="I36" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G36,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>1142513053</x:v>
+        <x:v>1175399124</x:v>
       </x:c>
       <x:c r="J36" s="43" t="n">
-        <x:f>IFERROR(I36/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.009137985631071913</x:v>
+        <x:f>IFERROR(I36/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.00940101321178211</x:v>
       </x:c>
       <x:c r="K36" s="31" t="n">
-        <x:f>RANK(I36,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I36,$I$9:$I$54,0)</x:f>
         <x:v>28</x:v>
       </x:c>
       <x:c r="L36" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G36,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="G37" s="30" t="str">
-        <x:v>Ninety One</x:v>
+        <x:v>T. Rowe Price</x:v>
       </x:c>
       <x:c r="H37" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G37,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>900000000</x:v>
+        <x:v>960000000</x:v>
       </x:c>
       <x:c r="I37" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G37,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>1077267573</x:v>
+        <x:v>1142513053</x:v>
       </x:c>
       <x:c r="J37" s="43" t="n">
-        <x:f>IFERROR(I37/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.008616142788955701</x:v>
+        <x:f>IFERROR(I37/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.009137985631071913</x:v>
       </x:c>
       <x:c r="K37" s="31" t="n">
-        <x:f>RANK(I37,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I37,$I$9:$I$54,0)</x:f>
         <x:v>29</x:v>
       </x:c>
       <x:c r="L37" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G37,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="G38" s="30" t="str">
-        <x:v>ClearBridge</x:v>
+        <x:v>Ninety One</x:v>
       </x:c>
       <x:c r="H38" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G38,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>760000000</x:v>
+        <x:v>900000000</x:v>
       </x:c>
       <x:c r="I38" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G38,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>1047858894</x:v>
+        <x:v>1077267573</x:v>
       </x:c>
       <x:c r="J38" s="43" t="n">
-        <x:f>IFERROR(I38/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.00838092789541452</x:v>
+        <x:f>IFERROR(I38/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.008616142788955701</x:v>
       </x:c>
       <x:c r="K38" s="31" t="n">
-        <x:f>RANK(I38,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I38,$I$9:$I$54,0)</x:f>
         <x:v>30</x:v>
       </x:c>
       <x:c r="L38" s="32" t="n">
@@ -32061,47 +30141,47 @@
     </x:row>
     <x:row r="39">
       <x:c r="G39" s="30" t="str">
-        <x:v>聯博</x:v>
+        <x:v>ClearBridge</x:v>
       </x:c>
       <x:c r="H39" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G39,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>900495639</x:v>
+        <x:v>760000000</x:v>
       </x:c>
       <x:c r="I39" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G39,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>897752897</x:v>
+        <x:v>1047858894</x:v>
       </x:c>
       <x:c r="J39" s="43" t="n">
-        <x:f>IFERROR(I39/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.007180358291310641</x:v>
+        <x:f>IFERROR(I39/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.00838092789541452</x:v>
       </x:c>
       <x:c r="K39" s="31" t="n">
-        <x:f>RANK(I39,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I39,$I$9:$I$54,0)</x:f>
         <x:v>31</x:v>
       </x:c>
       <x:c r="L39" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G39,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="G40" s="30" t="str">
-        <x:v>信安</x:v>
+        <x:v>聯博</x:v>
       </x:c>
       <x:c r="H40" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G40,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>708888643</x:v>
+        <x:v>900495639</x:v>
       </x:c>
       <x:c r="I40" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G40,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>801020312</x:v>
+        <x:v>897752897</x:v>
       </x:c>
       <x:c r="J40" s="43" t="n">
-        <x:f>IFERROR(I40/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.006406677002098759</x:v>
+        <x:f>IFERROR(I40/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.007180358291310641</x:v>
       </x:c>
       <x:c r="K40" s="31" t="n">
-        <x:f>RANK(I40,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I40,$I$9:$I$54,0)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="L40" s="32" t="n">
@@ -32111,197 +30191,197 @@
     </x:row>
     <x:row r="41">
       <x:c r="G41" s="30" t="str">
-        <x:v>Pictet</x:v>
+        <x:v>UBS</x:v>
       </x:c>
       <x:c r="H41" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G41,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>618843493</x:v>
+        <x:v>761201485</x:v>
       </x:c>
       <x:c r="I41" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G41,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>769778438</x:v>
+        <x:v>789561325</x:v>
       </x:c>
       <x:c r="J41" s="43" t="n">
-        <x:f>IFERROR(I41/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.00615679994822167</x:v>
+        <x:f>IFERROR(I41/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.0063150263568149375</x:v>
       </x:c>
       <x:c r="K41" s="31" t="n">
-        <x:f>RANK(I41,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I41,$I$9:$I$54,0)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="L41" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G41,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="G42" s="30" t="str">
-        <x:v>滙豐</x:v>
+        <x:v>Pictet</x:v>
       </x:c>
       <x:c r="H42" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G42,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>460000000</x:v>
+        <x:v>618843493</x:v>
       </x:c>
       <x:c r="I42" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G42,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>706462588</x:v>
+        <x:v>769778438</x:v>
       </x:c>
       <x:c r="J42" s="43" t="n">
-        <x:f>IFERROR(I42/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.005650390567602449</x:v>
+        <x:f>IFERROR(I42/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.00615679994822167</x:v>
       </x:c>
       <x:c r="K42" s="31" t="n">
-        <x:f>RANK(I42,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I42,$I$9:$I$54,0)</x:f>
         <x:v>34</x:v>
       </x:c>
       <x:c r="L42" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G42,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="G43" s="30" t="str">
-        <x:v>荷寶</x:v>
+        <x:v>滙豐</x:v>
       </x:c>
       <x:c r="H43" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G43,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>506416368</x:v>
+        <x:v>460000000</x:v>
       </x:c>
       <x:c r="I43" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G43,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>697308846</x:v>
+        <x:v>706462588</x:v>
       </x:c>
       <x:c r="J43" s="43" t="n">
-        <x:f>IFERROR(I43/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.005577177607236788</x:v>
+        <x:f>IFERROR(I43/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.005650390567602449</x:v>
       </x:c>
       <x:c r="K43" s="31" t="n">
-        <x:f>RANK(I43,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I43,$I$9:$I$54,0)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="L43" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G43,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="G44" s="30" t="str">
-        <x:v>摩根士丹利</x:v>
+        <x:v>荷寶</x:v>
       </x:c>
       <x:c r="H44" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G44,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>460000000</x:v>
+        <x:v>506416368</x:v>
       </x:c>
       <x:c r="I44" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G44,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>690570828</x:v>
+        <x:v>697308846</x:v>
       </x:c>
       <x:c r="J44" s="43" t="n">
-        <x:f>IFERROR(I44/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.005523285958905744</x:v>
+        <x:f>IFERROR(I44/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.005577177607236788</x:v>
       </x:c>
       <x:c r="K44" s="31" t="n">
-        <x:f>RANK(I44,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I44,$I$9:$I$54,0)</x:f>
         <x:v>36</x:v>
       </x:c>
       <x:c r="L44" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G44,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="G45" s="30" t="str">
-        <x:v>PGIM</x:v>
+        <x:v>摩根士丹利</x:v>
       </x:c>
       <x:c r="H45" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G45,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>600000000</x:v>
+        <x:v>460000000</x:v>
       </x:c>
       <x:c r="I45" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G45,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>688857784</x:v>
+        <x:v>690570828</x:v>
       </x:c>
       <x:c r="J45" s="43" t="n">
-        <x:f>IFERROR(I45/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.005509584783749547</x:v>
+        <x:f>IFERROR(I45/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.005523285958905744</x:v>
       </x:c>
       <x:c r="K45" s="31" t="n">
-        <x:f>RANK(I45,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I45,$I$9:$I$54,0)</x:f>
         <x:v>37</x:v>
       </x:c>
       <x:c r="L45" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G45,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="G46" s="30" t="str">
-        <x:v>Amundi</x:v>
+        <x:v>PGIM</x:v>
       </x:c>
       <x:c r="H46" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G46,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>500000000</x:v>
+        <x:v>600000000</x:v>
       </x:c>
       <x:c r="I46" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G46,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>666575819</x:v>
+        <x:v>688857784</x:v>
       </x:c>
       <x:c r="J46" s="43" t="n">
-        <x:f>IFERROR(I46/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.005331370385701836</x:v>
+        <x:f>IFERROR(I46/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.005509584783749547</x:v>
       </x:c>
       <x:c r="K46" s="31" t="n">
-        <x:f>RANK(I46,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I46,$I$9:$I$54,0)</x:f>
         <x:v>38</x:v>
       </x:c>
       <x:c r="L46" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G46,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="G47" s="30" t="str">
-        <x:v>LGIM</x:v>
+        <x:v>Amundi</x:v>
       </x:c>
       <x:c r="H47" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G47,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>400000000</x:v>
+        <x:v>500000000</x:v>
       </x:c>
       <x:c r="I47" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G47,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>593041556</x:v>
+        <x:v>666575819</x:v>
       </x:c>
       <x:c r="J47" s="43" t="n">
-        <x:f>IFERROR(I47/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.004743232651151627</x:v>
+        <x:f>IFERROR(I47/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.005331370385701836</x:v>
       </x:c>
       <x:c r="K47" s="31" t="n">
-        <x:f>RANK(I47,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I47,$I$9:$I$54,0)</x:f>
         <x:v>39</x:v>
       </x:c>
       <x:c r="L47" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G47,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="G48" s="30" t="str">
-        <x:v>信安環球</x:v>
+        <x:v>LGIM</x:v>
       </x:c>
       <x:c r="H48" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G48,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>425091462</x:v>
+        <x:v>400000000</x:v>
       </x:c>
       <x:c r="I48" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G48,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>478192278</x:v>
+        <x:v>593041556</x:v>
       </x:c>
       <x:c r="J48" s="43" t="n">
-        <x:f>IFERROR(I48/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.0038246514153861015</x:v>
+        <x:f>IFERROR(I48/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.004743232651151627</x:v>
       </x:c>
       <x:c r="K48" s="31" t="n">
-        <x:f>RANK(I48,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I48,$I$9:$I$54,0)</x:f>
         <x:v>40</x:v>
       </x:c>
       <x:c r="L48" s="32" t="n">
@@ -32322,11 +30402,11 @@
         <x:v>458409894</x:v>
       </x:c>
       <x:c r="J49" s="43" t="n">
-        <x:f>IFERROR(I49/SUM($I$9:$I$58),0)</x:f>
+        <x:f>IFERROR(I49/SUM($I$9:$I$54),0)</x:f>
         <x:v>0.0036664290298600195</x:v>
       </x:c>
       <x:c r="K49" s="31" t="n">
-        <x:f>RANK(I49,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I49,$I$9:$I$54,0)</x:f>
         <x:v>41</x:v>
       </x:c>
       <x:c r="L49" s="32" t="n">
@@ -32336,7 +30416,7 @@
     </x:row>
     <x:row r="50">
       <x:c r="G50" s="30" t="str">
-        <x:v>UBS</x:v>
+        <x:v>HSBC</x:v>
       </x:c>
       <x:c r="H50" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G50,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
@@ -32344,14 +30424,14 @@
       </x:c>
       <x:c r="I50" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G50,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>422040147</x:v>
+        <x:v>421747465</x:v>
       </x:c>
       <x:c r="J50" s="43" t="n">
-        <x:f>IFERROR(I50/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.0033755385016345</x:v>
+        <x:f>IFERROR(I50/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.003373197588413902</x:v>
       </x:c>
       <x:c r="K50" s="31" t="n">
-        <x:f>RANK(I50,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I50,$I$9:$I$54,0)</x:f>
         <x:v>42</x:v>
       </x:c>
       <x:c r="L50" s="32" t="n">
@@ -32361,22 +30441,22 @@
     </x:row>
     <x:row r="51">
       <x:c r="G51" s="30" t="str">
-        <x:v>HSBC</x:v>
+        <x:v>Allianz</x:v>
       </x:c>
       <x:c r="H51" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G51,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>400000000</x:v>
+        <x:v>275923278</x:v>
       </x:c>
       <x:c r="I51" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G51,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>421747465</x:v>
+        <x:v>275639320</x:v>
       </x:c>
       <x:c r="J51" s="43" t="n">
-        <x:f>IFERROR(I51/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.003373197588413902</x:v>
+        <x:f>IFERROR(I51/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0.002204603386284842</x:v>
       </x:c>
       <x:c r="K51" s="31" t="n">
-        <x:f>RANK(I51,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I51,$I$9:$I$54,0)</x:f>
         <x:v>43</x:v>
       </x:c>
       <x:c r="L51" s="32" t="n">
@@ -32386,176 +30466,76 @@
     </x:row>
     <x:row r="52">
       <x:c r="G52" s="30" t="str">
-        <x:v>瑞銀</x:v>
+        <x:v>柏瑞</x:v>
       </x:c>
       <x:c r="H52" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G52,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>361201485</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I52" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G52,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>367521178</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J52" s="43" t="n">
-        <x:f>IFERROR(I52/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.002939487855180437</x:v>
+        <x:f>IFERROR(I52/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K52" s="31" t="n">
-        <x:f>RANK(I52,$I$9:$I$58,0)</x:f>
+        <x:f>RANK(I52,$I$9:$I$54,0)</x:f>
         <x:v>44</x:v>
       </x:c>
       <x:c r="L52" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G52,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="G53" s="30" t="str">
-        <x:v>Allianz</x:v>
+        <x:v>玉山</x:v>
       </x:c>
       <x:c r="H53" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G53,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>275923278</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I53" s="40" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G53,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>275639320</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J53" s="43" t="n">
-        <x:f>IFERROR(I53/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0.002204603386284842</x:v>
+        <x:f>IFERROR(I53/SUM($I$9:$I$54),0)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K53" s="31" t="n">
-        <x:f>RANK(I53,$I$9:$I$58,0)</x:f>
-        <x:v>45</x:v>
+        <x:f>RANK(I53,$I$9:$I$54,0)</x:f>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="L53" s="32" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G53,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="G54" s="30" t="str">
-        <x:v>柏瑞</x:v>
-      </x:c>
-      <x:c r="H54" s="40" t="n">
+      <x:c r="G54" s="33" t="str">
+        <x:v>國泰</x:v>
+      </x:c>
+      <x:c r="H54" s="41" t="n">
         <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G54,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I54" s="40" t="n">
+      <x:c r="I54" s="41" t="n">
         <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G54,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J54" s="43" t="n">
-        <x:f>IFERROR(I54/SUM($I$9:$I$58),0)</x:f>
+      <x:c r="J54" s="44" t="n">
+        <x:f>IFERROR(I54/SUM($I$9:$I$54),0)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K54" s="31" t="n">
-        <x:f>RANK(I54,$I$9:$I$58,0)</x:f>
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="L54" s="32" t="n">
+      <x:c r="K54" s="34" t="n">
+        <x:f>RANK(I54,$I$9:$I$54,0)</x:f>
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="L54" s="35" t="n">
         <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G54,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="G55" s="30" t="str">
-        <x:v>安聯</x:v>
-      </x:c>
-      <x:c r="H55" s="40" t="n">
-        <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G55,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I55" s="40" t="n">
-        <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G55,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J55" s="43" t="n">
-        <x:f>IFERROR(I55/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K55" s="31" t="n">
-        <x:f>RANK(I55,$I$9:$I$58,0)</x:f>
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="L55" s="32" t="n">
-        <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G55,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="G56" s="30" t="str">
-        <x:v>玉山</x:v>
-      </x:c>
-      <x:c r="H56" s="40" t="n">
-        <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G56,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I56" s="40" t="n">
-        <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G56,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J56" s="43" t="n">
-        <x:f>IFERROR(I56/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K56" s="31" t="n">
-        <x:f>RANK(I56,$I$9:$I$58,0)</x:f>
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="L56" s="32" t="n">
-        <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G56,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57">
-      <x:c r="G57" s="30" t="str">
-        <x:v>野村</x:v>
-      </x:c>
-      <x:c r="H57" s="40" t="n">
-        <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G57,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I57" s="40" t="n">
-        <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G57,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J57" s="43" t="n">
-        <x:f>IFERROR(I57/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K57" s="31" t="n">
-        <x:f>RANK(I57,$I$9:$I$58,0)</x:f>
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="L57" s="32" t="n">
-        <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G57,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58">
-      <x:c r="G58" s="33" t="str">
-        <x:v>國泰</x:v>
-      </x:c>
-      <x:c r="H58" s="41" t="n">
-        <x:f>SUMIFS('國外委外明細'!$G$4:$G$188,'國外委外明細'!$F$4:$F$188,G58,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I58" s="41" t="n">
-        <x:f>SUMIFS('國外委外明細'!$H$4:$H$188,'國外委外明細'!$F$4:$F$188,G58,'國外委外明細'!$A$4:$A$188,$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J58" s="44" t="n">
-        <x:f>IFERROR(I58/SUM($I$9:$I$58),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K58" s="34" t="n">
-        <x:f>RANK(I58,$I$9:$I$58,0)</x:f>
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="L58" s="35" t="n">
-        <x:f>COUNTIFS('國外委外明細'!$F$4:$F$188,G58,'國外委外明細'!$A$4:$A$188,$B$4,'國外委外明細'!$J$4:$J$188,"&lt;&gt;解約")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32564,7 +30544,7 @@
     <x:mergeCell ref="A1:AB1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4068634ba3d4894"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45831a0033ca4cbf"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Separate self managed and delegated pie chart categories
</commit_message>
<xml_diff>
--- a/outputs/blf-monthly-disclosure/勞工退休基金月度揭露_可持續更新.xlsx
+++ b/outputs/blf-monthly-disclosure/勞工退休基金月度揭露_可持續更新.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板" sheetId="1" r:id="Rea57131bbd824ffa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板(美元)" sheetId="2" r:id="Rc7f6dd0ef8624f3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度資產配置" sheetId="3" r:id="R8f610c8024324425"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國內委外明細" sheetId="4" r:id="R503ecde672d34e62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國外委外明細" sheetId="5" r:id="R4ebe21c7b8d64aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次彙總" sheetId="6" r:id="R802666f003924e1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業者彙總" sheetId="7" r:id="R9c0fb9a211e949db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新說明" sheetId="8" r:id="Red807b104c3e47b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料品質檢核" sheetId="9" r:id="R435746bd90384b4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板" sheetId="1" r:id="R4818d5ca136d45d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板(美元)" sheetId="2" r:id="Rc7badedce6024dea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度資產配置" sheetId="3" r:id="R1ee838209b6846ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國內委外明細" sheetId="4" r:id="R386c6cba956148f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國外委外明細" sheetId="5" r:id="R0e1ce79a85344cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次彙總" sheetId="6" r:id="Rd6ea12b3b34e4f62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業者彙總" sheetId="7" r:id="R20c90765d3ce449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新說明" sheetId="8" r:id="R915d050253f44ea8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料品質檢核" sheetId="9" r:id="R857a65ef08204e5e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,10 +571,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$V$12:$V$15</c:f>
+              <c:f>'儀表板'!$V$12:$V$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -582,7 +618,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$W$12:$W$15</c:f>
+              <c:f>'儀表板'!$W$12:$W$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -673,10 +709,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$AD$12:$AD$15</c:f>
+              <c:f>'儀表板(美元)'!$AD$12:$AD$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -684,7 +756,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$AE$12:$AE$15</c:f>
+              <c:f>'儀表板(美元)'!$AE$12:$AE$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1517,10 +1589,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$X$12:$X$15</c:f>
+              <c:f>'儀表板'!$X$12:$X$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1528,7 +1636,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$Y$12:$Y$15</c:f>
+              <c:f>'儀表板'!$Y$12:$Y$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1619,10 +1727,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$Z$12:$Z$15</c:f>
+              <c:f>'儀表板'!$Z$12:$Z$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1630,7 +1774,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$AA$12:$AA$15</c:f>
+              <c:f>'儀表板'!$AA$12:$AA$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1721,10 +1865,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$AB$12:$AB$15</c:f>
+              <c:f>'儀表板'!$AB$12:$AB$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1732,7 +1912,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$AC$12:$AC$15</c:f>
+              <c:f>'儀表板'!$AC$12:$AC$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1823,10 +2003,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板'!$AD$12:$AD$15</c:f>
+              <c:f>'儀表板'!$AD$12:$AD$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1834,7 +2050,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板'!$AE$12:$AE$15</c:f>
+              <c:f>'儀表板'!$AE$12:$AE$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1925,10 +2141,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$V$12:$V$15</c:f>
+              <c:f>'儀表板(美元)'!$V$12:$V$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1936,7 +2188,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$W$12:$W$15</c:f>
+              <c:f>'儀表板(美元)'!$W$12:$W$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -2027,10 +2279,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$X$12:$X$15</c:f>
+              <c:f>'儀表板(美元)'!$X$12:$X$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -2038,7 +2326,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$Y$12:$Y$15</c:f>
+              <c:f>'儀表板(美元)'!$Y$12:$Y$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -2129,10 +2417,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$Z$12:$Z$15</c:f>
+              <c:f>'儀表板(美元)'!$Z$12:$Z$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -2140,7 +2464,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$AA$12:$AA$15</c:f>
+              <c:f>'儀表板(美元)'!$AA$12:$AA$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -2231,10 +2555,46 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+            </c:dLbl>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'儀表板(美元)'!$AB$12:$AB$15</c:f>
+              <c:f>'儀表板(美元)'!$AB$12:$AB$19</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -2242,7 +2602,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'儀表板(美元)'!$AC$12:$AC$15</c:f>
+              <c:f>'儀表板(美元)'!$AC$12:$AC$19</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -2295,7 +2655,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rddc8e118ed474418"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R499b756ae71d4727"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2325,7 +2685,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6b65fbf37bde4894"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd0e0e4b4a3044b20"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2355,7 +2715,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a329b0c78c647c2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R67a7b50753e84862"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2385,7 +2745,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b4a3c4fd0d84121"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R10fe982a9454461a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2415,7 +2775,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R55ef10ffbb394b03"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b77855f2a9843c4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2450,7 +2810,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb2a6c0d367bd46fa"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3ac6eea6adbd48dd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2480,7 +2840,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R56c9937843464ec6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R78f0ba3d51114af9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2510,7 +2870,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1c39af05f56c4eb8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R23039cf788e748e1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2540,7 +2900,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra0ea1935afa845af"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R818fabeb35b946c1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2570,7 +2930,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbe4c7fa4cb2f4027"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re0232fed47cc4d50"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2605,7 +2965,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca4d8f8b1ada4398"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f0ef1055a014989"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2635,7 +2995,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R19e78b81399f4313"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R736bb5eb73e54bd4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2665,7 +3025,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc4beec4e9e464d05"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra456163f163f4cb0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2695,7 +3055,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfce1f130435241f8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raeff7a0e2b9e498b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3291,39 +3651,39 @@
         <x:v>來源與報價時間已註明</x:v>
       </x:c>
       <x:c r="V12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="W12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.22060000000000002</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19999999999999998</x:v>
       </x:c>
       <x:c r="X12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="Y12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1165</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.4086</x:v>
       </x:c>
       <x:c r="Z12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="AA12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1724</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="AB12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="AC12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1711</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.3965</x:v>
       </x:c>
       <x:c r="AD12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="AE12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.45747499999999997</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.9830249999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -3351,39 +3711,39 @@
         <x:v>2654.12955439</x:v>
       </x:c>
       <x:c r="V13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="W13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.4739</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.12080000000000002</x:v>
       </x:c>
       <x:c r="X13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="Y13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.3744</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0248</x:v>
       </x:c>
       <x:c r="Z13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="AA13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.2375</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1151</x:v>
       </x:c>
       <x:c r="AB13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="AC13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.3722</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.12240000000000001</x:v>
       </x:c>
       <x:c r="AD13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="AE13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.8622749999999999</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.095775</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -3411,39 +3771,39 @@
         <x:v>802.98009492</x:v>
       </x:c>
       <x:c r="V14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="W14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1055</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.014100000000000001</x:v>
       </x:c>
       <x:c r="X14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="Y14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1005</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0184</x:v>
       </x:c>
       <x:c r="Z14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="AA14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.0901</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0604</x:v>
       </x:c>
       <x:c r="AB14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="AC14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.060200000000000004</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0668</x:v>
       </x:c>
       <x:c r="AD14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="AE14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.119375</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.039925</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -3471,39 +3831,39 @@
         <x:v>15244.879584</x:v>
       </x:c>
       <x:c r="V15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="W15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.19999999999999998</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.007700000000000001</x:v>
       </x:c>
       <x:c r="X15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="Y15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.4086</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Z15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="AA15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.5</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0067</x:v>
       </x:c>
       <x:c r="AB15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="AC15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.3965</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.026000000000000002</x:v>
       </x:c>
       <x:c r="AD15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="AE15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.9830249999999999</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.010100000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -3530,6 +3890,41 @@
         <x:f>SUM(B16:E16)</x:f>
         <x:v>8443.91807301</x:v>
       </x:c>
+      <x:c r="V16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="W16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19620000000000004</x:v>
+      </x:c>
+      <x:c r="X16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="Y16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.153</x:v>
+      </x:c>
+      <x:c r="Z16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AA16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.041299999999999996</x:v>
+      </x:c>
+      <x:c r="AB16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AC16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.11349999999999999</x:v>
+      </x:c>
+      <x:c r="AD16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AE16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.126</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="30" t="str">
@@ -3555,6 +3950,41 @@
         <x:f>SUM(B17:E17)</x:f>
         <x:v>22133.584103189998</x:v>
       </x:c>
+      <x:c r="V17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="W17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.09980000000000001</x:v>
+      </x:c>
+      <x:c r="X17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="Y17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0917</x:v>
+      </x:c>
+      <x:c r="Z17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="AA17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.057300000000000004</x:v>
+      </x:c>
+      <x:c r="AB17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="AC17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0487</x:v>
+      </x:c>
+      <x:c r="AD17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="AE17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.07437500000000001</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="30" t="str">
@@ -3580,6 +4010,41 @@
         <x:f>SUM(B18:E18)</x:f>
         <x:v>8729.960386230001</x:v>
       </x:c>
+      <x:c r="V18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="W18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.26360000000000006</x:v>
+      </x:c>
+      <x:c r="X18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="Y18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.203</x:v>
+      </x:c>
+      <x:c r="Z18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AA18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1358</x:v>
+      </x:c>
+      <x:c r="AB18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AC18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19190000000000002</x:v>
+      </x:c>
+      <x:c r="AD18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AE18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.198575</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="30" t="str">
@@ -3604,6 +4069,41 @@
       <x:c r="F19" s="66" t="n">
         <x:f>SUM(B19:E19)</x:f>
         <x:v>9274.65680763</x:v>
+      </x:c>
+      <x:c r="V19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="W19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.09780000000000001</x:v>
+      </x:c>
+      <x:c r="X19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="Y19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1005</x:v>
+      </x:c>
+      <x:c r="Z19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="AA19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0834</x:v>
+      </x:c>
+      <x:c r="AB19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="AC19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0342</x:v>
+      </x:c>
+      <x:c r="AD19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="AE19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.078975</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -3837,7 +4337,7 @@
     <x:mergeCell ref="A3:T3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e123d448f714b76"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2af10b403a8454d"/>
 </x:worksheet>
 </file>
 
@@ -4158,39 +4658,39 @@
         <x:v>來源與報價時間已註明</x:v>
       </x:c>
       <x:c r="V12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="W12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.22060000000000002</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19999999999999998</x:v>
       </x:c>
       <x:c r="X12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="Y12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1165</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.4086</x:v>
       </x:c>
       <x:c r="Z12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="AA12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1724</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="AB12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="AC12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1711</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.3965</x:v>
       </x:c>
       <x:c r="AD12" t="str">
-        <x:v>固定收益</x:v>
+        <x:v>自行運用 - 其他</x:v>
       </x:c>
       <x:c r="AE12" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.45747499999999997</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.9830249999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4218,39 +4718,39 @@
         <x:v>8.30843498009078</x:v>
       </x:c>
       <x:c r="V13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="W13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.4739</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.12080000000000002</x:v>
       </x:c>
       <x:c r="X13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="Y13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.3744</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0248</x:v>
       </x:c>
       <x:c r="Z13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="AA13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.2375</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1151</x:v>
       </x:c>
       <x:c r="AB13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="AC13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.3722</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.12240000000000001</x:v>
       </x:c>
       <x:c r="AD13" t="str">
-        <x:v>權益證券</x:v>
+        <x:v>自行運用 - 固定收益</x:v>
       </x:c>
       <x:c r="AE13" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.8622749999999999</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.095775</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4278,39 +4778,39 @@
         <x:v>2.513633103521678</x:v>
       </x:c>
       <x:c r="V14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="W14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1055</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.014100000000000001</x:v>
       </x:c>
       <x:c r="X14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="Y14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.1005</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0184</x:v>
       </x:c>
       <x:c r="Z14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="AA14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.0901</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0604</x:v>
       </x:c>
       <x:c r="AB14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="AC14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.060200000000000004</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0668</x:v>
       </x:c>
       <x:c r="AD14" t="str">
-        <x:v>另類投資</x:v>
+        <x:v>自行運用 - 權益證券</x:v>
       </x:c>
       <x:c r="AE14" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.119375</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.039925</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -4338,39 +4838,39 @@
         <x:v>47.7222713538895</x:v>
       </x:c>
       <x:c r="V15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="W15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.19999999999999998</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.007700000000000001</x:v>
       </x:c>
       <x:c r="X15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="Y15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.4086</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Z15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="AA15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.5</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0067</x:v>
       </x:c>
       <x:c r="AB15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="AC15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.3965</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.026000000000000002</x:v>
       </x:c>
       <x:c r="AD15" t="str">
-        <x:v>其他</x:v>
+        <x:v>自行運用 - 另類投資</x:v>
       </x:c>
       <x:c r="AE15" s="50" t="n">
-        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")),0)</x:f>
-        <x:v>0.9830249999999999</x:v>
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.010100000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -4397,6 +4897,41 @@
         <x:f>SUM(B16:E16)</x:f>
         <x:v>26.432675138550632</x:v>
       </x:c>
+      <x:c r="V16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="W16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19620000000000004</x:v>
+      </x:c>
+      <x:c r="X16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="Y16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.153</x:v>
+      </x:c>
+      <x:c r="Z16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AA16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.041299999999999996</x:v>
+      </x:c>
+      <x:c r="AB16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AC16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.11349999999999999</x:v>
+      </x:c>
+      <x:c r="AD16" t="str">
+        <x:v>國內委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AE16" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.126</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="30" t="str">
@@ -4422,6 +4957,41 @@
         <x:f>SUM(B17:E17)</x:f>
         <x:v>69.28653655717639</x:v>
       </x:c>
+      <x:c r="V17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="W17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.09980000000000001</x:v>
+      </x:c>
+      <x:c r="X17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="Y17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0917</x:v>
+      </x:c>
+      <x:c r="Z17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="AA17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.057300000000000004</x:v>
+      </x:c>
+      <x:c r="AB17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="AC17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0487</x:v>
+      </x:c>
+      <x:c r="AD17" t="str">
+        <x:v>國外委託經營 - 固定收益</x:v>
+      </x:c>
+      <x:c r="AE17" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.07437500000000001</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="30" t="str">
@@ -4447,6 +5017,41 @@
         <x:f>SUM(B18:E18)</x:f>
         <x:v>27.32809637260917</x:v>
       </x:c>
+      <x:c r="V18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="W18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.26360000000000006</x:v>
+      </x:c>
+      <x:c r="X18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="Y18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.203</x:v>
+      </x:c>
+      <x:c r="Z18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AA18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1358</x:v>
+      </x:c>
+      <x:c r="AB18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AC18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.19190000000000002</x:v>
+      </x:c>
+      <x:c r="AD18" t="str">
+        <x:v>國外委託經營 - 權益證券</x:v>
+      </x:c>
+      <x:c r="AE18" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.198575</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="30" t="str">
@@ -4471,6 +5076,41 @@
       <x:c r="F19" s="75" t="n">
         <x:f>SUM(B19:E19)</x:f>
         <x:v>29.033203342087965</x:v>
+      </x:c>
+      <x:c r="V19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="W19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"新制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.09780000000000001</x:v>
+      </x:c>
+      <x:c r="X19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="Y19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"舊制",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.1005</x:v>
+      </x:c>
+      <x:c r="Z19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="AA19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"勞工保險",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0834</x:v>
+      </x:c>
+      <x:c r="AB19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="AC19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$C$4:$C$263,"國民年金",'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.0342</x:v>
+      </x:c>
+      <x:c r="AD19" t="str">
+        <x:v>國外委託經營 - 另類投資</x:v>
+      </x:c>
+      <x:c r="AE19" s="50" t="n">
+        <x:f>IFERROR(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")/(SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"轉存金融機構")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政策性貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"短期票券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、公司債、金融債券及特別股")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"公債、金融債券、公司債及證券化商品")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"房屋及土地")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"政府或公營事業貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"被保險人貸款")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"股票及受益憑證投資（含期貨）")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"自行運用-國外-另類投資")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國內-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-固定收益")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-權益證券")+SUMIFS('月度資產配置'!$F$4:$F$263,'月度資產配置'!$A$4:$A$263,$A$6,'月度資產配置'!$D$4:$D$263,"委託經營-國外-另類投資")),0)</x:f>
+        <x:v>0.078975</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -4701,7 +5341,7 @@
     <x:mergeCell ref="A22:F22"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R576dfdfedbb3494b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5403afd071214b54"/>
 </x:worksheet>
 </file>
 
@@ -11523,7 +12163,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55ff615b097e473d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebd52607121e48c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16562,7 +17202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e109314e2a44d04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2456ac98db94528"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24541,7 +25181,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6614b9a4d8354037"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1d5ec689dcb43ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28480,7 +29120,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R234131b6140b42c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R460c4c544131444f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30544,7 +31184,7 @@
     <x:mergeCell ref="A1:AB1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45831a0033ca4cbf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b9351d7950405e"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Apply blue and orange pie chart color groups
</commit_message>
<xml_diff>
--- a/outputs/blf-monthly-disclosure/勞工退休基金月度揭露_可持續更新.xlsx
+++ b/outputs/blf-monthly-disclosure/勞工退休基金月度揭露_可持續更新.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板" sheetId="1" r:id="R4818d5ca136d45d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板(美元)" sheetId="2" r:id="Rc7badedce6024dea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度資產配置" sheetId="3" r:id="R1ee838209b6846ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國內委外明細" sheetId="4" r:id="R386c6cba956148f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國外委外明細" sheetId="5" r:id="R0e1ce79a85344cfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次彙總" sheetId="6" r:id="Rd6ea12b3b34e4f62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業者彙總" sheetId="7" r:id="R20c90765d3ce449a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新說明" sheetId="8" r:id="R915d050253f44ea8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料品質檢核" sheetId="9" r:id="R857a65ef08204e5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板" sheetId="1" r:id="R3812a4dc4885464a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="儀表板(美元)" sheetId="2" r:id="Ra7b6409e80534c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度資產配置" sheetId="3" r:id="R1df0219790804d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國內委外明細" sheetId="4" r:id="R0fa5779b336c4701"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國外委外明細" sheetId="5" r:id="R1e85928260b8496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次彙總" sheetId="6" r:id="R8638dd1b2e6c436f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業者彙總" sheetId="7" r:id="Rda5d593f2f644463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新說明" sheetId="8" r:id="Rbd590052f5c54440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料品質檢核" sheetId="9" r:id="R385aba81dc294349"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2655,7 +2655,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R499b756ae71d4727"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1c02425c7763405f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2685,7 +2685,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd0e0e4b4a3044b20"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R85b6d07abc184071"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2715,7 +2715,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R67a7b50753e84862"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd685d74b5cdc4258"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2745,7 +2745,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R10fe982a9454461a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9932d27bef4f408f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2775,7 +2775,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b77855f2a9843c4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0fec2278ac39463c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2810,7 +2810,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3ac6eea6adbd48dd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbec2c5d1eb024a8e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2840,7 +2840,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R78f0ba3d51114af9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5535927a18bd425a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2870,7 +2870,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R23039cf788e748e1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0354150bd16c4667"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2900,7 +2900,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R818fabeb35b946c1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2e1d400215d14885"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2930,7 +2930,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re0232fed47cc4d50"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7d7731605b9c41bc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2965,7 +2965,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f0ef1055a014989"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R00ee71bb6a294ea1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2995,7 +2995,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R736bb5eb73e54bd4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R50a29c93ec7a4935"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3025,7 +3025,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra456163f163f4cb0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R71c6ae55c236430f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3055,7 +3055,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raeff7a0e2b9e498b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9ed78a9b4a8d44d5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3169,10 +3169,10 @@
         <a:srgbClr val="2F75B5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="F4B183"/>
+        <a:srgbClr val="1F4E79"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="F4B183"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="C55A11"/>
@@ -4337,7 +4337,7 @@
     <x:mergeCell ref="A3:T3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2af10b403a8454d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a4b1262333b466d"/>
 </x:worksheet>
 </file>
 
@@ -5341,7 +5341,7 @@
     <x:mergeCell ref="A22:F22"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5403afd071214b54"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea3ee92266764a2b"/>
 </x:worksheet>
 </file>
 
@@ -12163,7 +12163,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebd52607121e48c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reebcba79ece4414b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17202,7 +17202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2456ac98db94528"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R987db0bfe72f496d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25181,7 +25181,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1d5ec689dcb43ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b73035b34d6401a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29120,7 +29120,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R460c4c544131444f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e6bf0e5ad12484d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31184,7 +31184,7 @@
     <x:mergeCell ref="A1:AB1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b9351d7950405e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5427ddb105fe434e"/>
 </x:worksheet>
 </file>
 

</xml_diff>